<commit_message>
Daily pipeline 2026-09-08: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U47"/>
+  <dimension ref="A1:U48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,100 +541,100 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46273.435</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>303</v>
-      </c>
-      <c r="K2" t="n">
-        <v>869</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>303</v>
+      </c>
+      <c r="K3" t="n">
+        <v>869</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -653,29 +653,25 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -696,27 +692,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -737,32 +733,32 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -778,32 +774,32 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -819,20 +815,20 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
@@ -858,25 +854,29 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -899,21 +899,21 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -936,21 +936,21 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -973,21 +973,21 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1010,21 +1010,21 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1047,21 +1047,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1084,21 +1084,21 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1121,21 +1121,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1154,29 +1154,25 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1195,25 +1191,29 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1236,21 +1236,21 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1273,21 +1273,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1297,46 +1297,34 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K21" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1346,9 +1334,17 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K22" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
@@ -1357,116 +1353,104 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>736</v>
-      </c>
-      <c r="K23" t="n">
-        <v>736</v>
-      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K24" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="N24" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
@@ -1477,113 +1461,125 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K25" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>785</v>
+      </c>
+      <c r="K26" t="n">
+        <v>785</v>
+      </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="N26" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1594,67 +1590,55 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J27" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K27" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1664,9 +1648,17 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K28" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
@@ -1675,13 +1667,13 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1692,136 +1684,128 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>849</v>
-      </c>
-      <c r="K29" t="n">
-        <v>849</v>
-      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O29" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K30" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
+      <c r="N30" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1833,14 +1817,14 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K31" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
@@ -1850,13 +1834,13 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1867,124 +1851,120 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M32" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N32" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O32" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K32" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B33" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K33" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M33" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -1995,61 +1975,53 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K34" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O34" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2060,57 +2032,61 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K35" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
+      <c r="N35" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2121,37 +2097,37 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K36" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
@@ -2161,17 +2137,17 @@
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2182,11 +2158,9 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
@@ -2195,48 +2169,46 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K37" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2247,23 +2219,25 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B38" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2274,30 +2248,32 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K38" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
+      <c r="N38" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2308,65 +2284,57 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M39" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N39" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J39" t="n">
+        <v>603</v>
+      </c>
+      <c r="K39" t="n">
+        <v>603</v>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2377,12 +2345,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>N</t>
@@ -2390,48 +2356,54 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>585</v>
-      </c>
-      <c r="K40" t="n">
-        <v>869</v>
-      </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M40" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N40" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2442,11 +2414,11 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2455,7 +2427,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2471,7 +2443,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K41" t="n">
         <v>869</v>
@@ -2479,7 +2451,7 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
@@ -2489,14 +2461,14 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2507,11 +2479,11 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2520,7 +2492,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2539,17 +2511,17 @@
         <v>303</v>
       </c>
       <c r="K42" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -2561,7 +2533,7 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2572,11 +2544,11 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2585,7 +2557,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2609,7 +2581,7 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
@@ -2626,7 +2598,7 @@
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2637,10 +2609,12 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>N</t>
@@ -2648,54 +2622,48 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M44" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J44" t="n">
+        <v>303</v>
+      </c>
+      <c r="K44" t="n">
+        <v>585</v>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
       <c r="N44" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O44" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2706,57 +2674,65 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K45" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M45" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N45" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2767,25 +2743,23 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B46" t="inlineStr"/>
-      <c r="C46" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -2796,32 +2770,30 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K46" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2832,11 +2804,11 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2845,7 +2817,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2869,12 +2841,12 @@
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -2886,10 +2858,75 @@
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>303</v>
+      </c>
+      <c r="K48" t="n">
+        <v>869</v>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-10: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U48"/>
+  <dimension ref="A1:U49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46273.435</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -567,111 +567,115 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46273.435</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>303</v>
-      </c>
-      <c r="K3" t="n">
-        <v>869</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>303</v>
+      </c>
+      <c r="K4" t="n">
+        <v>869</v>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -690,29 +694,25 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -733,27 +733,27 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -774,32 +774,32 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -815,32 +815,32 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -856,20 +856,20 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -895,25 +895,29 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -936,21 +940,21 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -973,21 +977,21 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1010,21 +1014,21 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1047,21 +1051,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1084,21 +1088,21 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1121,21 +1125,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1158,21 +1162,21 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1191,29 +1195,25 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1232,25 +1232,29 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1273,21 +1277,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1310,21 +1314,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1334,46 +1338,34 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K22" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1383,9 +1375,17 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K23" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
@@ -1394,116 +1394,104 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>736</v>
-      </c>
-      <c r="K24" t="n">
-        <v>736</v>
-      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K25" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
@@ -1514,113 +1502,125 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K26" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>785</v>
+      </c>
+      <c r="K27" t="n">
+        <v>785</v>
+      </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="N27" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1631,67 +1631,55 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K28" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1701,9 +1689,17 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K29" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
@@ -1712,13 +1708,13 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1729,136 +1725,128 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>849</v>
-      </c>
-      <c r="K30" t="n">
-        <v>849</v>
-      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K31" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="N31" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1870,14 +1858,14 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K32" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
@@ -1887,13 +1875,13 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -1904,124 +1892,120 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M33" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N33" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O33" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K33" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B34" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K34" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M34" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2032,61 +2016,53 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K35" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O35" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2097,57 +2073,61 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K36" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="N36" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2158,37 +2138,37 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K37" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
@@ -2198,17 +2178,17 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2219,11 +2199,9 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
@@ -2232,48 +2210,46 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K38" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2284,23 +2260,25 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B39" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -2311,30 +2289,32 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K39" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
+      <c r="N39" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2345,65 +2325,57 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N40" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J40" t="n">
+        <v>603</v>
+      </c>
+      <c r="K40" t="n">
+        <v>603</v>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2414,12 +2386,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B41" t="inlineStr"/>
-      <c r="C41" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>N</t>
@@ -2427,48 +2397,54 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>585</v>
-      </c>
-      <c r="K41" t="n">
-        <v>869</v>
-      </c>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M41" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N41" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2479,11 +2455,11 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2492,7 +2468,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2508,7 +2484,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K42" t="n">
         <v>869</v>
@@ -2516,7 +2492,7 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
@@ -2526,14 +2502,14 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2544,11 +2520,11 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2557,7 +2533,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2576,17 +2552,17 @@
         <v>303</v>
       </c>
       <c r="K43" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -2598,7 +2574,7 @@
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2609,11 +2585,11 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2622,7 +2598,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2646,7 +2622,7 @@
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
@@ -2663,7 +2639,7 @@
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2674,10 +2650,12 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
+      <c r="C45" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>N</t>
@@ -2685,54 +2663,48 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M45" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J45" t="n">
+        <v>303</v>
+      </c>
+      <c r="K45" t="n">
+        <v>585</v>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
       <c r="N45" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O45" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2743,57 +2715,65 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K46" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M46" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O46" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2804,25 +2784,23 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B47" t="inlineStr"/>
-      <c r="C47" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2833,32 +2811,30 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K47" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2869,11 +2845,11 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2882,7 +2858,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2906,12 +2882,12 @@
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -2923,10 +2899,75 @@
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>303</v>
+      </c>
+      <c r="K49" t="n">
+        <v>869</v>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="U49" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-11: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U49"/>
+  <dimension ref="A1:U52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,26 +541,34 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>663</v>
+      </c>
+      <c r="K2" t="n">
+        <v>663</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -569,27 +577,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46273.435</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -608,45 +616,41 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>303</v>
-      </c>
-      <c r="K4" t="n">
-        <v>869</v>
-      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -655,27 +659,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -694,25 +698,29 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46273.435</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -731,41 +739,45 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>303</v>
+      </c>
+      <c r="K7" t="n">
+        <v>869</v>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -774,27 +786,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -813,34 +825,30 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -856,27 +864,27 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -897,27 +905,27 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -936,30 +944,34 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>AL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -973,25 +985,29 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1010,25 +1026,29 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1051,21 +1071,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1088,21 +1108,21 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1125,21 +1145,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1162,21 +1182,21 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1199,21 +1219,21 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1232,29 +1252,25 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1277,21 +1293,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1314,21 +1330,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1347,25 +1363,29 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1375,46 +1395,34 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K23" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1433,30 +1441,22 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0053-26</t>
@@ -1464,63 +1464,39 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>736</v>
-      </c>
-      <c r="K25" t="n">
-        <v>736</v>
-      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1536,10 +1512,10 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>435.8</v>
+        <v>661.7</v>
       </c>
       <c r="K26" t="n">
-        <v>435.8</v>
+        <v>661.7</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
@@ -1555,113 +1531,109 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J27" t="n">
-        <v>785</v>
-      </c>
-      <c r="K27" t="n">
-        <v>785</v>
-      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>736</v>
+      </c>
+      <c r="K28" t="n">
+        <v>736</v>
+      </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="N28" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1672,14 +1644,14 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1691,14 +1663,14 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>325.2</v>
+        <v>435.8</v>
       </c>
       <c r="K29" t="n">
-        <v>325.2</v>
+        <v>435.8</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
@@ -1708,13 +1680,13 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1725,60 +1697,76 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>785</v>
+      </c>
+      <c r="K30" t="n">
+        <v>785</v>
+      </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
+      <c r="N30" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0046-26</t>
@@ -1786,49 +1774,25 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>849</v>
-      </c>
-      <c r="K31" t="n">
-        <v>849</v>
-      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1839,14 +1803,14 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1858,14 +1822,14 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>857</v>
+        <v>325.2</v>
       </c>
       <c r="K32" t="n">
-        <v>867</v>
+        <v>325.2</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
@@ -1875,13 +1839,13 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -1892,14 +1856,14 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1909,17 +1873,9 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J33" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="K33" t="n">
-        <v>10.3</v>
-      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
@@ -1928,13 +1884,13 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -1945,20 +1901,18 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46234.89293981482</v>
+      </c>
+      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1977,35 +1931,35 @@
           <t>LMR</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M34" t="n">
-        <v>-90.17319999999999</v>
-      </c>
+      <c r="J34" t="n">
+        <v>849</v>
+      </c>
+      <c r="K34" t="n">
+        <v>849</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" s="2" t="n">
-        <v>46188</v>
+        <v>46234</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>46195</v>
+        <v>46243</v>
       </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2016,23 +1970,19 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -2043,10 +1993,10 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>777.7</v>
+        <v>857</v>
       </c>
       <c r="K35" t="n">
-        <v>777.7</v>
+        <v>867</v>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -2054,42 +2004,38 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -2100,95 +2046,97 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>125.4</v>
+        <v>10.3</v>
       </c>
       <c r="K36" t="n">
-        <v>155.9</v>
+        <v>10.3</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O36" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46119.48518518519</v>
-      </c>
-      <c r="B37" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>686</v>
-      </c>
-      <c r="K37" t="n">
-        <v>686</v>
-      </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M37" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2199,37 +2147,37 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>348.7</v>
+        <v>777.7</v>
       </c>
       <c r="K38" t="n">
-        <v>348.7</v>
+        <v>777.7</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
@@ -2237,19 +2185,15 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
+      <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2260,11 +2204,9 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46146.4284375</v>
+      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
@@ -2273,48 +2215,50 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>303</v>
+        <v>125.4</v>
       </c>
       <c r="K39" t="n">
-        <v>869</v>
+        <v>155.9</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" s="2" t="n">
-        <v>46068</v>
-      </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
+        <v>46146</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2325,7 +2269,7 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
@@ -2336,7 +2280,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2352,10 +2296,10 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>603</v>
+        <v>686</v>
       </c>
       <c r="K40" t="n">
-        <v>603</v>
+        <v>686</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
@@ -2365,17 +2309,17 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2386,7 +2330,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
@@ -2397,54 +2341,46 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M41" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N41" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O41" s="2" t="n">
-        <v>46065</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="K41" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2455,12 +2391,12 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46058.58436342593</v>
-      </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" s="2" t="n">
-        <v>46068</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>N</t>
@@ -2468,7 +2404,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2484,7 +2420,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>585</v>
+        <v>303</v>
       </c>
       <c r="K42" t="n">
         <v>869</v>
@@ -2492,7 +2428,7 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
@@ -2502,14 +2438,14 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>10'6" draft, 6 barges wide</t>
+          <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2520,25 +2456,23 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B43" t="inlineStr"/>
-      <c r="C43" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2549,32 +2483,30 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="K43" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2585,12 +2517,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>N</t>
@@ -2598,48 +2528,54 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>303</v>
-      </c>
-      <c r="K44" t="n">
-        <v>585</v>
-      </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M44" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N44" s="2" t="n">
-        <v>46050</v>
-      </c>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2650,11 +2586,11 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" s="2" t="n">
-        <v>46050</v>
+        <v>46068</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2663,7 +2599,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2679,32 +2615,32 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K45" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" s="2" t="n">
-        <v>46045</v>
+        <v>46061</v>
       </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2715,10 +2651,12 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
+      <c r="C46" s="2" t="n">
+        <v>46061</v>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>N</t>
@@ -2726,54 +2664,48 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M46" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J46" t="n">
+        <v>303</v>
+      </c>
+      <c r="K46" t="n">
+        <v>869</v>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O46" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46052</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2784,23 +2716,25 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2811,30 +2745,32 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K47" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
+      <c r="N47" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2845,11 +2781,11 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2858,7 +2794,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2877,17 +2813,17 @@
         <v>303</v>
       </c>
       <c r="K48" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -2899,7 +2835,7 @@
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2910,64 +2846,259 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M49" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N49" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K50" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>303</v>
+      </c>
+      <c r="K51" t="n">
+        <v>869</v>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
         <v>46033.86975694444</v>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" s="2" t="n">
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0106-26</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J49" t="n">
+      <c r="J52" t="n">
         <v>303</v>
       </c>
-      <c r="K49" t="n">
+      <c r="K52" t="n">
         <v>869</v>
       </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" s="2" t="n">
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr">
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
+      <c r="Q52" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
-      <c r="T49" t="inlineStr">
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="U52" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-12: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U52"/>
+  <dimension ref="A1:U54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,75 +541,71 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46275.97677083333</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>663</v>
-      </c>
-      <c r="K2" t="n">
-        <v>663</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46275.64165509259</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0099-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>303</v>
+      </c>
+      <c r="K3" t="n">
+        <v>869</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,39 +614,47 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46275.6390625</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0098-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>663</v>
+      </c>
+      <c r="K4" t="n">
+        <v>663</v>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -659,27 +663,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -706,21 +710,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46273.435</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -739,45 +743,41 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>303</v>
-      </c>
-      <c r="K7" t="n">
-        <v>869</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -786,27 +786,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46273.435</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -829,33 +829,41 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>303</v>
+      </c>
+      <c r="K9" t="n">
+        <v>869</v>
+      </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -864,27 +872,27 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -903,29 +911,25 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>TX, LA - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -946,32 +950,32 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -993,21 +997,21 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1028,32 +1032,32 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1067,25 +1071,29 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1104,25 +1112,29 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1145,21 +1157,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1182,21 +1194,21 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1219,21 +1231,21 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1256,21 +1268,21 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1293,21 +1305,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1330,21 +1342,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1363,29 +1375,25 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1408,21 +1416,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1441,25 +1449,29 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1482,21 +1494,21 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1506,46 +1518,34 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J26" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K26" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1564,65 +1564,49 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="K28" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O28" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
@@ -1633,25 +1617,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1661,17 +1641,9 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K29" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
@@ -1680,24 +1652,20 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
@@ -1708,7 +1676,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1728,30 +1696,30 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="K30" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>46251</v>
+        <v>46257</v>
       </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1762,113 +1730,137 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K31" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="K32" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -1882,102 +1874,82 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="K34" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O34" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1987,17 +1959,9 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J35" t="n">
-        <v>857</v>
-      </c>
-      <c r="K35" t="n">
-        <v>867</v>
-      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
@@ -2006,13 +1970,13 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2023,161 +1987,155 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="K36" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="N36" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.73908564815</v>
+      </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M37" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N37" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O37" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="J37" t="n">
+        <v>857</v>
+      </c>
+      <c r="K37" t="n">
+        <v>867</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="K38" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
@@ -2185,28 +2143,30 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B39" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
@@ -2215,50 +2175,54 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K39" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M39" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N39" s="2" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O39" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2269,7 +2233,7 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
@@ -2280,7 +2244,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2296,10 +2260,10 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K40" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
@@ -2307,19 +2271,15 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2330,7 +2290,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
@@ -2341,12 +2301,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2357,30 +2317,34 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K41" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="N41" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2391,25 +2355,23 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -2420,32 +2382,30 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K42" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2456,37 +2416,37 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K43" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
@@ -2496,17 +2456,17 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2517,9 +2477,11 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B44" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
@@ -2528,54 +2490,48 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M44" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J44" t="n">
+        <v>303</v>
+      </c>
+      <c r="K44" t="n">
+        <v>869</v>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
       <c r="N44" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O44" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2586,25 +2542,23 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2615,32 +2569,30 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K45" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2651,12 +2603,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B46" t="inlineStr"/>
-      <c r="C46" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>N</t>
@@ -2664,48 +2614,54 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>303</v>
-      </c>
-      <c r="K46" t="n">
-        <v>869</v>
-      </c>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M46" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N46" s="2" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O46" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2716,11 +2672,11 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2729,7 +2685,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2745,32 +2701,32 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K47" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2781,11 +2737,11 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2794,7 +2750,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2813,17 +2769,17 @@
         <v>303</v>
       </c>
       <c r="K48" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -2835,7 +2791,7 @@
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2846,10 +2802,12 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>N</t>
@@ -2857,54 +2815,48 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M49" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J49" t="n">
+        <v>303</v>
+      </c>
+      <c r="K49" t="n">
+        <v>585</v>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O49" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2915,23 +2867,25 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
+      <c r="C50" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -2942,30 +2896,32 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K50" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
+      <c r="N50" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2976,12 +2932,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B51" t="inlineStr"/>
-      <c r="C51" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>N</t>
@@ -2989,48 +2943,54 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J51" t="n">
-        <v>303</v>
-      </c>
-      <c r="K51" t="n">
-        <v>869</v>
-      </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M51" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N51" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -3041,25 +3001,23 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B52" t="inlineStr"/>
-      <c r="C52" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
@@ -3070,35 +3028,163 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K52" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" s="2" t="n">
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>303</v>
+      </c>
+      <c r="K53" t="n">
+        <v>869</v>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>303</v>
+      </c>
+      <c r="K54" t="n">
+        <v>869</v>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr">
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr">
+      <c r="Q54" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
-      <c r="T52" t="inlineStr">
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="U54" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-13: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U54"/>
+  <dimension ref="A1:U55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,105 +541,105 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>482</v>
+      </c>
+      <c r="K2" t="n">
+        <v>482</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>303</v>
-      </c>
-      <c r="K3" t="n">
-        <v>869</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46275.97677083333</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -650,10 +650,10 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K4" t="n">
-        <v>663</v>
+        <v>869</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
@@ -663,39 +663,47 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46275.64165509259</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0099-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>663</v>
+      </c>
+      <c r="K5" t="n">
+        <v>663</v>
+      </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -704,27 +712,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46275.6390625</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0098-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -751,21 +759,21 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -792,21 +800,21 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46273.435</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -825,111 +833,115 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46273.435</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>303</v>
-      </c>
-      <c r="K9" t="n">
-        <v>869</v>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>303</v>
+      </c>
+      <c r="K10" t="n">
+        <v>869</v>
+      </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -948,29 +960,25 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -991,27 +999,27 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1032,32 +1040,32 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1073,32 +1081,32 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1114,20 +1122,20 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
@@ -1153,25 +1161,29 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1194,21 +1206,21 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1231,21 +1243,21 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1268,21 +1280,21 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1305,21 +1317,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1342,21 +1354,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1379,21 +1391,21 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1416,21 +1428,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1449,29 +1461,25 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1490,25 +1498,29 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1531,21 +1543,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1568,21 +1580,21 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1592,46 +1604,34 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K28" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1641,9 +1641,17 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K29" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
@@ -1652,116 +1660,104 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>736</v>
-      </c>
-      <c r="K30" t="n">
-        <v>736</v>
-      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K31" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="N31" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
@@ -1772,113 +1768,125 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K32" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O32" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>785</v>
+      </c>
+      <c r="K33" t="n">
+        <v>785</v>
+      </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="N33" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -1889,67 +1897,55 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J34" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K34" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1959,9 +1955,17 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K35" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
@@ -1970,13 +1974,13 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -1987,136 +1991,128 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J36" t="n">
-        <v>849</v>
-      </c>
-      <c r="K36" t="n">
-        <v>849</v>
-      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O36" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K37" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="N37" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2128,14 +2124,14 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K38" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
@@ -2145,13 +2141,13 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2162,124 +2158,120 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M39" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N39" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K39" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B40" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K40" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M40" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2290,61 +2282,53 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K41" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O41" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2355,57 +2339,61 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K42" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="N42" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2416,37 +2404,37 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K43" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
@@ -2456,17 +2444,17 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2477,11 +2465,9 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B44" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
@@ -2490,48 +2476,46 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K44" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2542,23 +2526,25 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B45" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2569,30 +2555,32 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K45" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
+      <c r="N45" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2603,65 +2591,57 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M46" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N46" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O46" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J46" t="n">
+        <v>603</v>
+      </c>
+      <c r="K46" t="n">
+        <v>603</v>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2672,12 +2652,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B47" t="inlineStr"/>
-      <c r="C47" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>N</t>
@@ -2685,48 +2663,54 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>585</v>
-      </c>
-      <c r="K47" t="n">
-        <v>869</v>
-      </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M47" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N47" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2737,11 +2721,11 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2750,7 +2734,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2766,7 +2750,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K48" t="n">
         <v>869</v>
@@ -2774,7 +2758,7 @@
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
@@ -2784,14 +2768,14 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2802,11 +2786,11 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2815,7 +2799,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2834,17 +2818,17 @@
         <v>303</v>
       </c>
       <c r="K49" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
       <c r="N49" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -2856,7 +2840,7 @@
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2867,11 +2851,11 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2880,7 +2864,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2904,7 +2888,7 @@
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
@@ -2921,7 +2905,7 @@
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2932,10 +2916,12 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
           <t>N</t>
@@ -2943,54 +2929,48 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M51" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J51" t="n">
+        <v>303</v>
+      </c>
+      <c r="K51" t="n">
+        <v>585</v>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
       <c r="N51" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O51" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -3001,57 +2981,65 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J52" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K52" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M52" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -3062,25 +3050,23 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B53" t="inlineStr"/>
-      <c r="C53" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -3091,32 +3077,30 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K53" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3127,11 +3111,11 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3140,7 +3124,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3164,12 +3148,12 @@
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
       <c r="N54" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -3181,10 +3165,75 @@
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>303</v>
+      </c>
+      <c r="K55" t="n">
+        <v>869</v>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="U55" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-14: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U55"/>
+  <dimension ref="A1:U57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,34 +541,26 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46279.4325</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>CGD-H BNM 0100-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>482</v>
-      </c>
-      <c r="K2" t="n">
-        <v>482</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -577,69 +569,81 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>303</v>
+      </c>
+      <c r="K3" t="n">
+        <v>869</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -650,10 +654,10 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>303</v>
+        <v>482</v>
       </c>
       <c r="K4" t="n">
-        <v>869</v>
+        <v>482</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
@@ -669,82 +673,78 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46275.97677083333</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>663</v>
-      </c>
-      <c r="K5" t="n">
-        <v>663</v>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46275.64165509259</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0099-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>303</v>
+      </c>
+      <c r="K6" t="n">
+        <v>869</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -753,39 +753,47 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46275.6390625</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0098-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>663</v>
+      </c>
+      <c r="K7" t="n">
+        <v>663</v>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -794,27 +802,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -841,21 +849,21 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46273.435</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -874,45 +882,41 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>303</v>
-      </c>
-      <c r="K10" t="n">
-        <v>869</v>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
@@ -921,27 +925,27 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46273.435</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -964,33 +968,41 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>303</v>
+      </c>
+      <c r="K12" t="n">
+        <v>869</v>
+      </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -999,27 +1011,27 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1038,29 +1050,25 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>TX, LA - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1081,32 +1089,32 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1128,21 +1136,21 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1163,32 +1171,32 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1202,25 +1210,29 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1239,25 +1251,29 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1280,21 +1296,21 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1317,21 +1333,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1354,21 +1370,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1391,21 +1407,21 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1428,21 +1444,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1465,21 +1481,21 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1498,29 +1514,25 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1543,21 +1555,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1576,25 +1588,29 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1617,21 +1633,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1641,46 +1657,34 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K29" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1699,65 +1703,49 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="K31" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
@@ -1768,25 +1756,21 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1796,17 +1780,9 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J32" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K32" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
@@ -1815,24 +1791,20 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
@@ -1843,7 +1815,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1863,30 +1835,30 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="K33" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" s="2" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>46251</v>
+        <v>46257</v>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -1897,113 +1869,137 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K34" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="K35" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
+      <c r="N35" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -2017,102 +2013,82 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="K37" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O37" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2122,17 +2098,9 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>857</v>
-      </c>
-      <c r="K38" t="n">
-        <v>867</v>
-      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
@@ -2141,13 +2109,13 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2158,161 +2126,155 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="K39" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="N39" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.73908564815</v>
+      </c>
+      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N40" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="J40" t="n">
+        <v>857</v>
+      </c>
+      <c r="K40" t="n">
+        <v>867</v>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="K41" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
@@ -2320,28 +2282,30 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B42" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
@@ -2350,50 +2314,54 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K42" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M42" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N42" s="2" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O42" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2404,7 +2372,7 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
@@ -2415,7 +2383,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2431,10 +2399,10 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K43" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
@@ -2442,19 +2410,15 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2465,7 +2429,7 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
@@ -2476,12 +2440,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -2492,30 +2456,34 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K44" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="N44" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2526,25 +2494,23 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B45" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2555,32 +2521,30 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K45" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2591,37 +2555,37 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K46" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
@@ -2631,17 +2595,17 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2652,9 +2616,11 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B47" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
@@ -2663,54 +2629,48 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M47" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J47" t="n">
+        <v>303</v>
+      </c>
+      <c r="K47" t="n">
+        <v>869</v>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
       <c r="N47" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O47" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2721,25 +2681,23 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B48" t="inlineStr"/>
-      <c r="C48" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
@@ -2750,32 +2708,30 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K48" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2786,12 +2742,10 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B49" t="inlineStr"/>
-      <c r="C49" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>N</t>
@@ -2799,48 +2753,54 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>303</v>
-      </c>
-      <c r="K49" t="n">
-        <v>869</v>
-      </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M49" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N49" s="2" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2851,11 +2811,11 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2864,7 +2824,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2880,32 +2840,32 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K50" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2916,11 +2876,11 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2929,7 +2889,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2948,17 +2908,17 @@
         <v>303</v>
       </c>
       <c r="K51" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -2970,7 +2930,7 @@
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2981,10 +2941,12 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
+      <c r="C52" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
           <t>N</t>
@@ -2992,54 +2954,48 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M52" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J52" t="n">
+        <v>303</v>
+      </c>
+      <c r="K52" t="n">
+        <v>585</v>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
       <c r="N52" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O52" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -3050,23 +3006,25 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -3077,30 +3035,32 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K53" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3111,12 +3071,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B54" t="inlineStr"/>
-      <c r="C54" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>N</t>
@@ -3124,48 +3082,54 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J54" t="n">
-        <v>303</v>
-      </c>
-      <c r="K54" t="n">
-        <v>869</v>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M54" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N54" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3176,25 +3140,23 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -3205,35 +3167,163 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K55" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" s="2" t="n">
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>303</v>
+      </c>
+      <c r="K56" t="n">
+        <v>869</v>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>303</v>
+      </c>
+      <c r="K57" t="n">
+        <v>869</v>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr">
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr">
+      <c r="Q57" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
-      <c r="T55" t="inlineStr">
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="U57" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-15: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U57"/>
+  <dimension ref="A1:U62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,26 +541,34 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46279.4325</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0100-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>691</v>
+      </c>
+      <c r="K2" t="n">
+        <v>701</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -569,47 +577,39 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46280.37981481481</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>CGD-H BNM 0104-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>303</v>
-      </c>
-      <c r="K3" t="n">
-        <v>869</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,47 +618,39 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>MS - LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER AND IPANEMA IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46280.37956018518</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>CGD-H BNM 0103-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>482</v>
-      </c>
-      <c r="K4" t="n">
-        <v>482</v>
-      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -667,27 +659,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>FL - GULF OF AMERICA - APALACHEE BAY</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>ON SEPTEMBER 16, 2026, FROM 1830Z UNTIL 2030Z, USAF PERSONNEL AIRDROPS WILL BE CONDUCTED IN APALACHEE BAY, WITHIN A 5 MILE RADIUS OF APPROXIMATE POSITION 29-55-00N 084-00-00W. MARINERS SHOULD AVOID THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//162130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46280.37930555556</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0102-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -706,45 +698,41 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//050500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46279.67928240741</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>CGD-H BNM 0101-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>303</v>
-      </c>
-      <c r="K6" t="n">
-        <v>869</v>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -753,47 +741,39 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>THE USAF WILL CONDUCT TESTS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA FROM 1200Z TO 1800Z, DAILY. THE HAZARD AREA IS BOUND BY APPROXIMATE POSITIONS: 30-09-55N 086-45-20W, 30-09-55N 086-37-16W, 30-03-08N 086-37-16W AND 30-03-08N 086-45-20W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//181900Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46275.97677083333</v>
+        <v>46279.4325</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>CGD-H BNM 0100-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>663</v>
-      </c>
-      <c r="K7" t="n">
-        <v>663</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -802,39 +782,47 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46275.64165509259</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0099-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>303</v>
+      </c>
+      <c r="K8" t="n">
+        <v>869</v>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
@@ -843,39 +831,47 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46275.6390625</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0098-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>482</v>
+      </c>
+      <c r="K9" t="n">
+        <v>482</v>
+      </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -884,27 +880,27 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -923,71 +919,79 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46273.435</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>303</v>
+      </c>
+      <c r="K11" t="n">
+        <v>869</v>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -998,10 +1002,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>303</v>
+        <v>663</v>
       </c>
       <c r="K12" t="n">
-        <v>869</v>
+        <v>663</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1011,27 +1015,27 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1050,25 +1054,29 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1089,27 +1097,27 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1130,27 +1138,27 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46273.435</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1169,41 +1177,45 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>303</v>
+      </c>
+      <c r="K17" t="n">
+        <v>869</v>
+      </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
@@ -1212,27 +1224,27 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1251,29 +1263,25 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>SEC LMR</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1292,25 +1300,29 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1329,25 +1341,29 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1366,30 +1382,34 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>AL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1403,25 +1423,29 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1440,25 +1464,29 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1481,21 +1509,21 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1518,21 +1546,21 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1555,21 +1583,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1588,29 +1616,25 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1633,21 +1657,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1670,21 +1694,21 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1707,21 +1731,21 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1731,46 +1755,34 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K31" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1791,92 +1803,64 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J33" t="n">
-        <v>736</v>
-      </c>
-      <c r="K33" t="n">
-        <v>736</v>
-      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O33" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1886,156 +1870,120 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J34" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K34" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J35" t="n">
-        <v>785</v>
-      </c>
-      <c r="K35" t="n">
-        <v>785</v>
-      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O35" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Osceola Harbor</t>
-        </is>
-      </c>
+      <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K36" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2045,17 +1993,9 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K37" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
@@ -2064,426 +2004,400 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>736</v>
+      </c>
+      <c r="K38" t="n">
+        <v>736</v>
+      </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="N38" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>849</v>
+        <v>435.8</v>
       </c>
       <c r="K39" t="n">
-        <v>849</v>
+        <v>435.8</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>857</v>
+        <v>785</v>
       </c>
       <c r="K40" t="n">
-        <v>867</v>
+        <v>785</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="N40" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="K41" t="n">
-        <v>10.3</v>
-      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46239.68305555556</v>
+      </c>
+      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M42" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N42" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O42" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K42" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J43" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K43" t="n">
-        <v>777.7</v>
-      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>125.4</v>
+        <v>849</v>
       </c>
       <c r="K44" t="n">
-        <v>155.9</v>
+        <v>849</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" s="2" t="n">
-        <v>46146</v>
+        <v>46234</v>
       </c>
       <c r="O44" s="2" t="n">
-        <v>46188</v>
+        <v>46243</v>
       </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2494,23 +2408,19 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2521,10 +2431,10 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>686</v>
+        <v>857</v>
       </c>
       <c r="K45" t="n">
-        <v>686</v>
+        <v>867</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
@@ -2534,44 +2444,36 @@
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -2582,10 +2484,10 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>348.7</v>
+        <v>10.3</v>
       </c>
       <c r="K46" t="n">
-        <v>348.7</v>
+        <v>10.3</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
@@ -2595,31 +2497,27 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>"Possible shoaling," transit area with caution</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46065.67140046296</v>
+        <v>46186.8905787037</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>46070</v>
+        <v>46199</v>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
@@ -2629,48 +2527,54 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>303</v>
-      </c>
-      <c r="K47" t="n">
-        <v>869</v>
-      </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M47" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N47" s="2" t="n">
-        <v>46068</v>
-      </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
+        <v>46188</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2681,7 +2585,7 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
@@ -2692,7 +2596,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2708,10 +2612,10 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>603</v>
+        <v>777.7</v>
       </c>
       <c r="K48" t="n">
-        <v>603</v>
+        <v>777.7</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
@@ -2719,11 +2623,7 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
+      <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr">
         <is>
           <t>Proceed with caution</t>
@@ -2731,7 +2631,7 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2742,7 +2642,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
@@ -2753,54 +2653,50 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M49" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>125.4</v>
+      </c>
+      <c r="K49" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" s="2" t="n">
-        <v>46062</v>
+        <v>46146</v>
       </c>
       <c r="O49" s="2" t="n">
-        <v>46065</v>
+        <v>46188</v>
       </c>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2811,25 +2707,23 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B50" t="inlineStr"/>
-      <c r="C50" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -2840,32 +2734,30 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>585</v>
+        <v>686</v>
       </c>
       <c r="K50" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2876,12 +2768,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B51" t="inlineStr"/>
-      <c r="C51" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>N</t>
@@ -2889,48 +2779,46 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K51" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
-      <c r="N51" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2941,12 +2829,12 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46050.44465277778</v>
-      </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" s="2" t="n">
-        <v>46052</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>N</t>
@@ -2954,7 +2842,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2973,17 +2861,17 @@
         <v>303</v>
       </c>
       <c r="K52" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" s="2" t="n">
-        <v>46050</v>
+        <v>46068</v>
       </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -2995,7 +2883,7 @@
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -3006,25 +2894,23 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B53" t="inlineStr"/>
-      <c r="C53" s="2" t="n">
-        <v>46050</v>
-      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -3035,32 +2921,30 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="K53" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3071,7 +2955,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
@@ -3082,7 +2966,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3104,32 +2988,32 @@
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="n">
-        <v>35.0859560963022</v>
+        <v>35.085769</v>
       </c>
       <c r="M54" t="n">
-        <v>-90.10785143484679</v>
+        <v>-90.10947400000001</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46062</v>
       </c>
       <c r="O54" s="2" t="n">
-        <v>46044</v>
+        <v>46065</v>
       </c>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
+          <t>Amrize Dock on Mckellar Lake</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3140,23 +3024,25 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -3167,30 +3053,32 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="K55" t="n">
-        <v>538.7</v>
+        <v>869</v>
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
+      <c r="N55" s="2" t="n">
+        <v>46061</v>
+      </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>10'6" draft, 6 barges wide</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3201,11 +3089,11 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" s="2" t="n">
-        <v>46045</v>
+        <v>46061</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3214,7 +3102,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3238,7 +3126,7 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" s="2" t="n">
-        <v>46037</v>
+        <v>46052</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
@@ -3255,7 +3143,7 @@
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3266,11 +3154,11 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" s="2" t="n">
-        <v>46037</v>
+        <v>46052</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -3279,7 +3167,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3298,17 +3186,17 @@
         <v>303</v>
       </c>
       <c r="K57" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
       <c r="N57" s="2" t="n">
-        <v>46034</v>
+        <v>46050</v>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -3320,10 +3208,335 @@
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>303</v>
+      </c>
+      <c r="K58" t="n">
+        <v>585</v>
+      </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M59" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O59" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K60" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>303</v>
+      </c>
+      <c r="K61" t="n">
+        <v>869</v>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>303</v>
+      </c>
+      <c r="K62" t="n">
+        <v>869</v>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="U62" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-16: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U62"/>
+  <dimension ref="A1:U63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,75 +541,71 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>691</v>
-      </c>
-      <c r="K2" t="n">
-        <v>701</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46280.37981481481</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0104-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>691</v>
+      </c>
+      <c r="K3" t="n">
+        <v>701</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,27 +614,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>MS - LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER AND IPANEMA IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//010500Z OCT 26// BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46280.37956018518</v>
+        <v>46280.37981481481</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0103-26</t>
+          <t>CGD-H BNM 0104-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -659,27 +655,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA - APALACHEE BAY</t>
+          <t>MS - LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>ON SEPTEMBER 16, 2026, FROM 1830Z UNTIL 2030Z, USAF PERSONNEL AIRDROPS WILL BE CONDUCTED IN APALACHEE BAY, WITHIN A 5 MILE RADIUS OF APPROXIMATE POSITION 29-55-00N 084-00-00W. MARINERS SHOULD AVOID THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//162130Z SEP 26// BT</t>
+          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER AND IPANEMA IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46280.37930555556</v>
+        <v>46280.37956018518</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0102-26</t>
+          <t>CGD-H BNM 0103-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -700,27 +696,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA - APALACHEE BAY</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//050500Z OCT 26// BT</t>
+          <t>ON SEPTEMBER 16, 2026, FROM 1830Z UNTIL 2030Z, USAF PERSONNEL AIRDROPS WILL BE CONDUCTED IN APALACHEE BAY, WITHIN A 5 MILE RADIUS OF APPROXIMATE POSITION 29-55-00N 084-00-00W. MARINERS SHOULD AVOID THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//162130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46279.67928240741</v>
+        <v>46280.37930555556</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0101-26</t>
+          <t>CGD-H BNM 0102-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -747,21 +743,21 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>THE USAF WILL CONDUCT TESTS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA FROM 1200Z TO 1800Z, DAILY. THE HAZARD AREA IS BOUND BY APPROXIMATE POSITIONS: 30-09-55N 086-45-20W, 30-09-55N 086-37-16W, 30-03-08N 086-37-16W AND 30-03-08N 086-45-20W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//181900Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//050500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46279.4325</v>
+        <v>46279.67928240741</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0100-26</t>
+          <t>CGD-H BNM 0101-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -782,47 +778,39 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
+          <t>THE USAF WILL CONDUCT TESTS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA FROM 1200Z TO 1800Z, DAILY. THE HAZARD AREA IS BOUND BY APPROXIMATE POSITIONS: 30-09-55N 086-45-20W, 30-09-55N 086-37-16W, 30-03-08N 086-37-16W AND 30-03-08N 086-45-20W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//181900Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46279.4325</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>CGD-H BNM 0100-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>303</v>
-      </c>
-      <c r="K8" t="n">
-        <v>869</v>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
@@ -831,32 +819,32 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -867,10 +855,10 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>482</v>
+        <v>303</v>
       </c>
       <c r="K9" t="n">
-        <v>482</v>
+        <v>869</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
@@ -886,112 +874,112 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>482</v>
+      </c>
+      <c r="K10" t="n">
+        <v>482</v>
+      </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>303</v>
-      </c>
-      <c r="K11" t="n">
-        <v>869</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46275.97677083333</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1002,10 +990,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K12" t="n">
-        <v>663</v>
+        <v>869</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1015,39 +1003,47 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46275.64165509259</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0099-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>663</v>
+      </c>
+      <c r="K13" t="n">
+        <v>663</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1056,27 +1052,27 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46275.6390625</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0098-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1103,21 +1099,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1144,21 +1140,21 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46273.435</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1177,111 +1173,115 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46273.435</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>303</v>
-      </c>
-      <c r="K17" t="n">
-        <v>869</v>
-      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>303</v>
+      </c>
+      <c r="K18" t="n">
+        <v>869</v>
+      </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1300,29 +1300,25 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1343,27 +1339,27 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1384,32 +1380,32 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1425,32 +1421,32 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1466,20 +1462,20 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
@@ -1505,25 +1501,29 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1546,21 +1546,21 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1583,21 +1583,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1620,21 +1620,21 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1657,21 +1657,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1694,21 +1694,21 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1731,21 +1731,21 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1768,21 +1768,21 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1801,29 +1801,25 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1842,25 +1838,29 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1883,21 +1883,21 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1920,21 +1920,21 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1944,46 +1944,34 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J36" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K36" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1993,9 +1981,17 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K37" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
@@ -2004,116 +2000,104 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>736</v>
-      </c>
-      <c r="K38" t="n">
-        <v>736</v>
-      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O38" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K39" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="N39" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
@@ -2124,113 +2108,125 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K40" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>785</v>
+      </c>
+      <c r="K41" t="n">
+        <v>785</v>
+      </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="N41" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2241,67 +2237,55 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K42" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2311,9 +2295,17 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K43" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
@@ -2322,13 +2314,13 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2339,136 +2331,128 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J44" t="n">
-        <v>849</v>
-      </c>
-      <c r="K44" t="n">
-        <v>849</v>
-      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O44" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K45" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+      <c r="N45" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2480,14 +2464,14 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K46" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
@@ -2497,13 +2481,13 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2514,124 +2498,120 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B47" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M47" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N47" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O47" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B48" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K48" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M48" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2642,61 +2622,53 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K49" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O49" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2707,57 +2679,61 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K50" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="N50" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2768,37 +2744,37 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K51" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
@@ -2808,17 +2784,17 @@
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2829,11 +2805,9 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B52" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
@@ -2842,48 +2816,46 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K52" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -2894,23 +2866,25 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B53" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -2921,30 +2895,32 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K53" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -2955,65 +2931,57 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M54" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N54" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O54" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J54" t="n">
+        <v>603</v>
+      </c>
+      <c r="K54" t="n">
+        <v>603</v>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3024,12 +2992,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>N</t>
@@ -3037,48 +3003,54 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J55" t="n">
-        <v>585</v>
-      </c>
-      <c r="K55" t="n">
-        <v>869</v>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M55" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N55" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3089,11 +3061,11 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3102,7 +3074,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3118,7 +3090,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K56" t="n">
         <v>869</v>
@@ -3126,7 +3098,7 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
@@ -3136,14 +3108,14 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3154,11 +3126,11 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -3167,7 +3139,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3186,17 +3158,17 @@
         <v>303</v>
       </c>
       <c r="K57" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
       <c r="N57" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -3208,7 +3180,7 @@
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -3219,11 +3191,11 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3232,7 +3204,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3256,7 +3228,7 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
       <c r="N58" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
@@ -3273,7 +3245,7 @@
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -3284,10 +3256,12 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>N</t>
@@ -3295,54 +3269,48 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M59" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J59" t="n">
+        <v>303</v>
+      </c>
+      <c r="K59" t="n">
+        <v>585</v>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
       <c r="N59" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O59" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S59" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -3353,57 +3321,65 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J60" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K60" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M60" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -3414,25 +3390,23 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -3443,32 +3417,30 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K61" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q61" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -3479,11 +3451,11 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3492,7 +3464,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3516,12 +3488,12 @@
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
       <c r="N62" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -3533,10 +3505,75 @@
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>303</v>
+      </c>
+      <c r="K63" t="n">
+        <v>869</v>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="U63" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-17: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U63"/>
+  <dimension ref="A1:U65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,71 +541,75 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46281.41737268519</v>
+        <v>46281.77060185185</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>652</v>
+      </c>
+      <c r="K2" t="n">
+        <v>652</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46281.54202546296</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>CGD-H BNM 0105-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>691</v>
-      </c>
-      <c r="K3" t="n">
-        <v>701</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -614,27 +618,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>FROM 18SEP2026 TO 21SEP2026, BETWEEN 2300Z AND 0400Z, THE FOLLOWING DAY, THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-17-03N 086-24-47W,30-16-54N 086-11-14W,30-12-36N 085-59-45W,30-01-32N 085-48-15W,29-40-17N 085-48-36W,29-31-25N 085-59-27W,29-27-30N 086-17-51W,29-32-03N 086-36-18W,29-42-00N 086-46-25W,30-01-24N 086-46-35W AND30-12-38N 086-38-28W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46280.37981481481</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0104-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -653,41 +657,45 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>MS - LA - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER AND IPANEMA IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//010500Z OCT 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46280.37956018518</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0103-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>691</v>
+      </c>
+      <c r="K5" t="n">
+        <v>701</v>
+      </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -696,27 +704,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA - APALACHEE BAY</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>ON SEPTEMBER 16, 2026, FROM 1830Z UNTIL 2030Z, USAF PERSONNEL AIRDROPS WILL BE CONDUCTED IN APALACHEE BAY, WITHIN A 5 MILE RADIUS OF APPROXIMATE POSITION 29-55-00N 084-00-00W. MARINERS SHOULD AVOID THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//162130Z SEP 26// BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46280.37930555556</v>
+        <v>46280.37981481481</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0102-26</t>
+          <t>CGD-H BNM 0104-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -737,27 +745,27 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>MS - LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//050500Z OCT 26// BT</t>
+          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER AND IPANEMA IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46279.67928240741</v>
+        <v>46280.37956018518</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0101-26</t>
+          <t>CGD-H BNM 0103-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -778,27 +786,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA - APALACHEE BAY</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>THE USAF WILL CONDUCT TESTS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA FROM 1200Z TO 1800Z, DAILY. THE HAZARD AREA IS BOUND BY APPROXIMATE POSITIONS: 30-09-55N 086-45-20W, 30-09-55N 086-37-16W, 30-03-08N 086-37-16W AND 30-03-08N 086-45-20W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//181900Z SEP 26// BT</t>
+          <t>ON SEPTEMBER 16, 2026, FROM 1830Z UNTIL 2030Z, USAF PERSONNEL AIRDROPS WILL BE CONDUCTED IN APALACHEE BAY, WITHIN A 5 MILE RADIUS OF APPROXIMATE POSITION 29-55-00N 084-00-00W. MARINERS SHOULD AVOID THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//162130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46279.4325</v>
+        <v>46280.37930555556</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0100-26</t>
+          <t>CGD-H BNM 0102-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -819,47 +827,39 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
+          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//050500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46279.67928240741</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>CGD-H BNM 0101-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>303</v>
-      </c>
-      <c r="K9" t="n">
-        <v>869</v>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -868,47 +868,39 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>THE USAF WILL CONDUCT TESTS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA FROM 1200Z TO 1800Z, DAILY. THE HAZARD AREA IS BOUND BY APPROXIMATE POSITIONS: 30-09-55N 086-45-20W, 30-09-55N 086-37-16W, 30-03-08N 086-37-16W AND 30-03-08N 086-45-20W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//181900Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46279.4325</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>CGD-H BNM 0100-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>482</v>
-      </c>
-      <c r="K10" t="n">
-        <v>482</v>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
@@ -917,69 +909,81 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>303</v>
+      </c>
+      <c r="K11" t="n">
+        <v>869</v>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -990,10 +994,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>303</v>
+        <v>482</v>
       </c>
       <c r="K12" t="n">
-        <v>869</v>
+        <v>482</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1009,82 +1013,78 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46275.97677083333</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>663</v>
-      </c>
-      <c r="K13" t="n">
-        <v>663</v>
-      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46275.64165509259</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0099-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>303</v>
+      </c>
+      <c r="K14" t="n">
+        <v>869</v>
+      </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
@@ -1093,39 +1093,47 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46275.6390625</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0098-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>663</v>
+      </c>
+      <c r="K15" t="n">
+        <v>663</v>
+      </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
@@ -1134,27 +1142,27 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1181,21 +1189,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46273.435</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1214,45 +1222,41 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>303</v>
-      </c>
-      <c r="K18" t="n">
-        <v>869</v>
-      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
@@ -1261,27 +1265,27 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46273.435</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1304,33 +1308,41 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>303</v>
+      </c>
+      <c r="K20" t="n">
+        <v>869</v>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
@@ -1339,27 +1351,27 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1378,29 +1390,25 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>TX, LA - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1421,32 +1429,32 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1468,21 +1476,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1503,32 +1511,32 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1542,25 +1550,29 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1579,25 +1591,29 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1620,21 +1636,21 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1657,21 +1673,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1694,21 +1710,21 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1731,21 +1747,21 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1768,21 +1784,21 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1805,21 +1821,21 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1838,29 +1854,25 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1883,21 +1895,21 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1916,25 +1928,29 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1957,21 +1973,21 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1981,46 +1997,34 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K37" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2039,65 +2043,49 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="K39" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
@@ -2108,25 +2096,21 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2136,17 +2120,9 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J40" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K40" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
@@ -2155,24 +2131,20 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
@@ -2183,7 +2155,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2203,30 +2175,30 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="K41" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" s="2" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O41" s="2" t="n">
-        <v>46251</v>
+        <v>46257</v>
       </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2237,113 +2209,137 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K42" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="K43" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="N43" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -2357,102 +2353,82 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="K45" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O45" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2462,17 +2438,9 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J46" t="n">
-        <v>857</v>
-      </c>
-      <c r="K46" t="n">
-        <v>867</v>
-      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -2481,13 +2449,13 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2498,161 +2466,155 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="K47" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
+      <c r="N47" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.73908564815</v>
+      </c>
+      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M48" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N48" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O48" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="J48" t="n">
+        <v>857</v>
+      </c>
+      <c r="K48" t="n">
+        <v>867</v>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="K49" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
@@ -2660,28 +2622,30 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B50" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
@@ -2690,50 +2654,54 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J50" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K50" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M50" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N50" s="2" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O50" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2744,7 +2712,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
@@ -2755,7 +2723,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2771,10 +2739,10 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K51" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
@@ -2782,19 +2750,15 @@
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2805,7 +2769,7 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
@@ -2816,12 +2780,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
@@ -2832,30 +2796,34 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K52" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="N52" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -2866,25 +2834,23 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B53" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -2895,32 +2861,30 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K53" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -2931,37 +2895,37 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K54" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
@@ -2971,17 +2935,17 @@
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -2992,9 +2956,11 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B55" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
@@ -3003,54 +2969,48 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M55" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J55" t="n">
+        <v>303</v>
+      </c>
+      <c r="K55" t="n">
+        <v>869</v>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
       <c r="N55" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O55" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3061,25 +3021,23 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B56" t="inlineStr"/>
-      <c r="C56" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -3090,32 +3048,30 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K56" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q56" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3126,12 +3082,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B57" t="inlineStr"/>
-      <c r="C57" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>N</t>
@@ -3139,48 +3093,54 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J57" t="n">
-        <v>303</v>
-      </c>
-      <c r="K57" t="n">
-        <v>869</v>
-      </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M57" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N57" s="2" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O57" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -3191,11 +3151,11 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3204,7 +3164,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3220,32 +3180,32 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K58" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
       <c r="N58" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -3256,11 +3216,11 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3269,7 +3229,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3288,17 +3248,17 @@
         <v>303</v>
       </c>
       <c r="K59" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
       <c r="N59" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -3310,7 +3270,7 @@
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -3321,10 +3281,12 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
           <t>N</t>
@@ -3332,54 +3294,48 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M60" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J60" t="n">
+        <v>303</v>
+      </c>
+      <c r="K60" t="n">
+        <v>585</v>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
       <c r="N60" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O60" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S60" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -3390,23 +3346,25 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -3417,30 +3375,32 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K61" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+      <c r="N61" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S61" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -3451,12 +3411,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B62" t="inlineStr"/>
-      <c r="C62" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>N</t>
@@ -3464,48 +3422,54 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J62" t="n">
-        <v>303</v>
-      </c>
-      <c r="K62" t="n">
-        <v>869</v>
-      </c>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M62" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N62" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O62" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -3516,25 +3480,23 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B63" t="inlineStr"/>
-      <c r="C63" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
@@ -3545,35 +3507,163 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K63" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
-      <c r="N63" s="2" t="n">
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>303</v>
+      </c>
+      <c r="K64" t="n">
+        <v>869</v>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>303</v>
+      </c>
+      <c r="K65" t="n">
+        <v>869</v>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr">
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="Q65" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
-      <c r="T63" t="inlineStr">
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="U65" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-18: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U65"/>
+  <dimension ref="A1:U66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46281.77060185185</v>
+        <v>46282.57303240741</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -564,10 +564,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>652</v>
+        <v>691</v>
       </c>
       <c r="K2" t="n">
-        <v>652</v>
+        <v>701.2</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
@@ -583,33 +583,41 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46281.54202546296</v>
+        <v>46281.77060185185</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0105-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>652</v>
+      </c>
+      <c r="K3" t="n">
+        <v>652</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,27 +626,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>FROM 18SEP2026 TO 21SEP2026, BETWEEN 2300Z AND 0400Z, THE FOLLOWING DAY, THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-17-03N 086-24-47W,30-16-54N 086-11-14W,30-12-36N 085-59-45W,30-01-32N 085-48-15W,29-40-17N 085-48-36W,29-31-25N 085-59-27W,29-27-30N 086-17-51W,29-32-03N 086-36-18W,29-42-00N 086-46-25W,30-01-24N 086-46-35W AND30-12-38N 086-38-28W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46281.41737268519</v>
+        <v>46281.54202546296</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>CGD-H BNM 0105-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -657,86 +665,86 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>FROM 18SEP2026 TO 21SEP2026, BETWEEN 2300Z AND 0400Z, THE FOLLOWING DAY, THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-17-03N 086-24-47W,30-16-54N 086-11-14W,30-12-36N 085-59-45W,30-01-32N 085-48-15W,29-40-17N 085-48-36W,29-31-25N 085-59-27W,29-27-30N 086-17-51W,29-32-03N 086-36-18W,29-42-00N 086-46-25W,30-01-24N 086-46-35W AND30-12-38N 086-38-28W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>691</v>
-      </c>
-      <c r="K5" t="n">
-        <v>701</v>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46280.37981481481</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0104-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>691</v>
+      </c>
+      <c r="K6" t="n">
+        <v>701</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -745,27 +753,27 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>MS - LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER AND IPANEMA IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//010500Z OCT 26// BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46280.37956018518</v>
+        <v>46280.37981481481</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0103-26</t>
+          <t>CGD-H BNM 0104-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -786,27 +794,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA - APALACHEE BAY</t>
+          <t>MS - LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>ON SEPTEMBER 16, 2026, FROM 1830Z UNTIL 2030Z, USAF PERSONNEL AIRDROPS WILL BE CONDUCTED IN APALACHEE BAY, WITHIN A 5 MILE RADIUS OF APPROXIMATE POSITION 29-55-00N 084-00-00W. MARINERS SHOULD AVOID THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//162130Z SEP 26// BT</t>
+          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER AND IPANEMA IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46280.37930555556</v>
+        <v>46280.37956018518</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0102-26</t>
+          <t>CGD-H BNM 0103-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -827,27 +835,27 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA - APALACHEE BAY</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//050500Z OCT 26// BT</t>
+          <t>ON SEPTEMBER 16, 2026, FROM 1830Z UNTIL 2030Z, USAF PERSONNEL AIRDROPS WILL BE CONDUCTED IN APALACHEE BAY, WITHIN A 5 MILE RADIUS OF APPROXIMATE POSITION 29-55-00N 084-00-00W. MARINERS SHOULD AVOID THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//162130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46279.67928240741</v>
+        <v>46280.37930555556</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0101-26</t>
+          <t>CGD-H BNM 0102-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -874,21 +882,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>THE USAF WILL CONDUCT TESTS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA FROM 1200Z TO 1800Z, DAILY. THE HAZARD AREA IS BOUND BY APPROXIMATE POSITIONS: 30-09-55N 086-45-20W, 30-09-55N 086-37-16W, 30-03-08N 086-37-16W AND 30-03-08N 086-45-20W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//181900Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//050500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46279.4325</v>
+        <v>46279.67928240741</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0100-26</t>
+          <t>CGD-H BNM 0101-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -909,47 +917,39 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
+          <t>THE USAF WILL CONDUCT TESTS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA FROM 1200Z TO 1800Z, DAILY. THE HAZARD AREA IS BOUND BY APPROXIMATE POSITIONS: 30-09-55N 086-45-20W, 30-09-55N 086-37-16W, 30-03-08N 086-37-16W AND 30-03-08N 086-45-20W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//181900Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46279.4325</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>CGD-H BNM 0100-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>303</v>
-      </c>
-      <c r="K11" t="n">
-        <v>869</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
@@ -958,32 +958,32 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>DIVING OPERATIONS ARE TAKING PLACE DURING DAYLIGHT HOURSFROM THE M/V NOBLE GLOBETROTTER 2 IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-51-18N 090-07-30W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//052359Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -994,10 +994,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>482</v>
+        <v>303</v>
       </c>
       <c r="K12" t="n">
-        <v>482</v>
+        <v>869</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1013,112 +1013,112 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>482</v>
+      </c>
+      <c r="K13" t="n">
+        <v>482</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>303</v>
-      </c>
-      <c r="K14" t="n">
-        <v>869</v>
-      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46275.97677083333</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1129,10 +1129,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K15" t="n">
-        <v>663</v>
+        <v>869</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1142,39 +1142,47 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46275.64165509259</v>
+        <v>46275.97677083333</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0099-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>663</v>
+      </c>
+      <c r="K16" t="n">
+        <v>663</v>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1183,27 +1191,27 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46275.6390625</v>
+        <v>46275.64165509259</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0098-26</t>
+          <t>CGD-H BNM 0099-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1230,21 +1238,21 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV MC40 WITHIN 20MILES OF APPROXIMATE POSITION 28-11-27.59N 088-29-45.59W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46274.60354166666</v>
+        <v>46275.6390625</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0097-26</t>
+          <t>CGD-H BNM 0098-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1271,21 +1279,21 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA BY THE USV SP-48, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-20-25N 089-24-28W,28-20-25N 088-51-18W,27-47-07N 088-51-18W AND27-47-07N 089-24-28W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV.CANCEL AT//210500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46273.435</v>
+        <v>46274.60354166666</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0097-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1304,111 +1312,115 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>AN 8 FT UNLIT YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 28-37-18N 090-34-06W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//160500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46273.435</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>303</v>
-      </c>
-      <c r="K20" t="n">
-        <v>869</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>303</v>
+      </c>
+      <c r="K21" t="n">
+        <v>869</v>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1427,29 +1439,25 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1470,27 +1478,27 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1511,32 +1519,32 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1552,32 +1560,32 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1593,20 +1601,20 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
@@ -1632,25 +1640,29 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1673,21 +1685,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1710,21 +1722,21 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1747,21 +1759,21 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1784,21 +1796,21 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1821,21 +1833,21 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1858,21 +1870,21 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1895,21 +1907,21 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1928,29 +1940,25 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1969,25 +1977,29 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2010,21 +2022,21 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2047,21 +2059,21 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2071,46 +2083,34 @@
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K39" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2120,9 +2120,17 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K40" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
@@ -2131,116 +2139,104 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
-        <v>736</v>
-      </c>
-      <c r="K41" t="n">
-        <v>736</v>
-      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O41" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K42" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="N42" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
@@ -2251,113 +2247,125 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K43" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O43" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>785</v>
+      </c>
+      <c r="K44" t="n">
+        <v>785</v>
+      </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="N44" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2368,67 +2376,55 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J45" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K45" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2438,9 +2434,17 @@
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K46" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -2449,13 +2453,13 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2466,136 +2470,128 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>849</v>
-      </c>
-      <c r="K47" t="n">
-        <v>849</v>
-      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O47" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K48" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="N48" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S48" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2607,14 +2603,14 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K49" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
@@ -2624,13 +2620,13 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2641,124 +2637,120 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M50" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N50" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O50" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K50" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B51" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J51" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K51" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M51" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2769,61 +2761,53 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K52" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O52" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -2834,57 +2818,61 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K53" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+      <c r="N53" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -2895,37 +2883,37 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K54" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
@@ -2935,17 +2923,17 @@
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -2956,11 +2944,9 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B55" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
@@ -2969,48 +2955,46 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K55" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3021,23 +3005,25 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B56" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -3048,30 +3034,32 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K56" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
+      <c r="N56" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S56" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3082,65 +3070,57 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M57" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N57" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O57" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J57" t="n">
+        <v>603</v>
+      </c>
+      <c r="K57" t="n">
+        <v>603</v>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -3151,12 +3131,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B58" t="inlineStr"/>
-      <c r="C58" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>N</t>
@@ -3164,48 +3142,54 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J58" t="n">
-        <v>585</v>
-      </c>
-      <c r="K58" t="n">
-        <v>869</v>
-      </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M58" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N58" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O58" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -3216,11 +3200,11 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3229,7 +3213,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3245,7 +3229,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K59" t="n">
         <v>869</v>
@@ -3253,7 +3237,7 @@
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
       <c r="N59" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
@@ -3263,14 +3247,14 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -3281,11 +3265,11 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3294,7 +3278,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3313,17 +3297,17 @@
         <v>303</v>
       </c>
       <c r="K60" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
       <c r="N60" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -3335,7 +3319,7 @@
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -3346,11 +3330,11 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3359,7 +3343,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3383,7 +3367,7 @@
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
       <c r="N61" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
@@ -3400,7 +3384,7 @@
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -3411,10 +3395,12 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>N</t>
@@ -3422,54 +3408,48 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M62" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J62" t="n">
+        <v>303</v>
+      </c>
+      <c r="K62" t="n">
+        <v>585</v>
+      </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
       <c r="N62" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O62" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -3480,57 +3460,65 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J63" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K63" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M63" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N63" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O63" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -3541,25 +3529,23 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B64" t="inlineStr"/>
-      <c r="C64" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
@@ -3570,32 +3556,30 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K64" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
-      <c r="N64" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q64" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
@@ -3606,11 +3590,11 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3619,7 +3603,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3643,12 +3627,12 @@
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
       <c r="N65" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -3660,10 +3644,75 @@
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>303</v>
+      </c>
+      <c r="K66" t="n">
+        <v>869</v>
+      </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="U66" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Restyle draft restriction hover box: bold section labels on own lines, sentence-based wrapping, larger font for draft-depth line
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malcor\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BAC8FC-0B1E-4FEC-B9F0-49217CDC495D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A9EA52-27C8-44FD-8DAC-43AD1E222DA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -484,13 +484,13 @@
     <t>n</t>
   </si>
   <si>
-    <t>Draft shall not exceed 10'6". Barge configurations not to exceed 4 wide and 6 long max on loads. Barge configurations not to exceed 6 wide and 7 long overall</t>
-  </si>
-  <si>
-    <t>Draft not to exceed 11'6". Barge configurations not to exceed 7 wide.</t>
-  </si>
-  <si>
-    <t>Barge drafts not to exceed 12'6". Barge configurations not to exceed 7 wide.</t>
+    <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+  </si>
+  <si>
+    <t>11'6" draft. 7 barges wide.</t>
+  </si>
+  <si>
+    <t>12'6" draft. 7 barges wide.</t>
   </si>
 </sst>
 </file>
@@ -498,7 +498,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -556,14 +556,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -969,10 +968,10 @@
       <c r="K2">
         <v>701.2</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="4">
         <v>46277</v>
       </c>
-      <c r="O2" s="5">
+      <c r="O2" s="4">
         <v>46283</v>
       </c>
       <c r="S2" t="s">
@@ -1010,10 +1009,10 @@
       <c r="K3">
         <v>652</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="4">
         <v>46281</v>
       </c>
-      <c r="O3" s="5">
+      <c r="O3" s="4">
         <v>46287</v>
       </c>
       <c r="S3" t="s">
@@ -1071,7 +1070,7 @@
       <c r="K5">
         <v>701</v>
       </c>
-      <c r="N5" s="5"/>
+      <c r="N5" s="4"/>
       <c r="T5" t="s">
         <v>31</v>
       </c>
@@ -1101,6 +1100,9 @@
       <c r="K6">
         <v>869</v>
       </c>
+      <c r="N6" s="4">
+        <v>46278</v>
+      </c>
       <c r="P6" t="s">
         <v>154</v>
       </c>
@@ -1136,6 +1138,9 @@
       <c r="K7">
         <v>585</v>
       </c>
+      <c r="N7" s="4">
+        <v>46278</v>
+      </c>
       <c r="P7" t="s">
         <v>154</v>
       </c>
@@ -1222,7 +1227,7 @@
       <c r="A11" s="2">
         <v>46275.976770833331</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>46291</v>
       </c>
       <c r="D11" t="s">
@@ -1246,10 +1251,10 @@
       <c r="K11">
         <v>663</v>
       </c>
-      <c r="N11" s="5">
+      <c r="N11" s="4">
         <v>46275</v>
       </c>
-      <c r="O11" s="5">
+      <c r="O11" s="4">
         <v>46281</v>
       </c>
       <c r="T11" t="s">

</xml_diff>

<commit_message>
Stop daily pipeline from collapsing manually split notice rows
fetch_notices.py deduped the whole notices sheet on (message_id,
date_published), which deleted intentional per-segment splits of one
notice. Now only incoming rows whose key already exists are skipped.
Restores the LMR 303-585 row of SEC LMR BNM 0058-26 UPDATE-1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,118 +417,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U54"/>
+  <dimension ref="A1:U55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>date_published</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>cancelled_date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>replaced_date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>active?</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>message_id</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>other_notes</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>dredge</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>river</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>mm_low</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>mm_high</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>lon</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>date_start</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>date_end</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>northbound</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>southbound</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>location_details</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>instructions</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>full_memo</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46286.49263888889</v>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -581,7 +569,7 @@
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46283.70012731481</v>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -622,7 +610,7 @@
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46283.699375</v>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -671,7 +659,7 @@
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46282.57303240741</v>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -710,10 +698,10 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="1" t="n">
         <v>46277</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="O5" s="1" t="n">
         <v>46283</v>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -736,7 +724,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46281.77060185185</v>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -775,10 +763,10 @@
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="1" t="n">
         <v>46281</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="O6" s="1" t="n">
         <v>46287</v>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -801,7 +789,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46281.41737268519</v>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -842,7 +830,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46280.38037037037</v>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -903,7 +891,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>46278.72424768518</v>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -938,7 +926,7 @@
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" s="2" t="n">
+      <c r="N9" s="1" t="n">
         <v>46278</v>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -966,8 +954,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>46277.53633101852</v>
+      <c r="A10" s="1" t="n">
+        <v>46278.72424768518</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -978,12 +966,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -994,22 +982,32 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>482</v>
+        <v>303</v>
       </c>
       <c r="K10" t="n">
-        <v>482</v>
+        <v>585</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" s="1" t="n">
+        <v>46278</v>
+      </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>12'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1019,27 +1017,39 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>46277.09849537037</v>
+      <c r="A11" s="1" t="n">
+        <v>46277.53633101852</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>482</v>
+      </c>
+      <c r="K11" t="n">
+        <v>482</v>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
@@ -1050,41 +1060,37 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr"/>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>46276.67863425926</v>
+      <c r="A12" s="1" t="n">
+        <v>46277.09849537037</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>303</v>
-      </c>
-      <c r="K12" t="n">
-        <v>869</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -1095,111 +1101,115 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>46275.97677083333</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>46291</v>
-      </c>
+      <c r="A13" s="1" t="n">
+        <v>46276.67863425926</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K13" t="n">
-        <v>663</v>
+        <v>869</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>46281</v>
-      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>n</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>46273.435</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="A14" s="1" t="n">
+        <v>46275.97677083333</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46291</v>
+      </c>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>663</v>
+      </c>
+      <c r="K14" t="n">
+        <v>663</v>
+      </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="N14" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O14" s="1" t="n">
+        <v>46281</v>
+      </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1209,39 +1219,27 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>46268.97141203703</v>
+      <c r="A15" s="1" t="n">
+        <v>46273.435</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>303</v>
-      </c>
-      <c r="K15" t="n">
-        <v>869</v>
-      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
@@ -1252,37 +1250,49 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>46268.53527777778</v>
+      <c r="A16" s="1" t="n">
+        <v>46268.97141203703</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>303</v>
+      </c>
+      <c r="K16" t="n">
+        <v>869</v>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1293,21 +1303,25 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr"/>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>46265.53005787037</v>
+      <c r="A17" s="1" t="n">
+        <v>46268.53527777778</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1330,14 +1344,14 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>46265.52835648148</v>
+      <c r="A18" s="1" t="n">
+        <v>46265.53005787037</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -1367,21 +1381,21 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>46265.52792824074</v>
+      <c r="A19" s="1" t="n">
+        <v>46265.52835648148</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1404,21 +1418,21 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>46265.52664351852</v>
+      <c r="A20" s="1" t="n">
+        <v>46265.52792824074</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1441,21 +1455,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>46265.52623842593</v>
+      <c r="A21" s="1" t="n">
+        <v>46265.52664351852</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1478,21 +1492,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>46265.52559027778</v>
+      <c r="A22" s="1" t="n">
+        <v>46265.52623842593</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1515,21 +1529,21 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>46265.52508101852</v>
+      <c r="A23" s="1" t="n">
+        <v>46265.52559027778</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1552,21 +1566,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>46265.52371527778</v>
+      <c r="A24" s="1" t="n">
+        <v>46265.52508101852</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1589,21 +1603,21 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>46258.44554398148</v>
+      <c r="A25" s="1" t="n">
+        <v>46265.52371527778</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1626,21 +1640,21 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>46258.44363425926</v>
+      <c r="A26" s="1" t="n">
+        <v>46258.44554398148</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1663,21 +1677,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>46257.8184375</v>
+      <c r="A27" s="1" t="n">
+        <v>46258.44363425926</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1700,21 +1714,21 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>46255.75466435185</v>
+      <c r="A28" s="1" t="n">
+        <v>46257.8184375</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1724,50 +1738,34 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K28" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>46253.46241898148</v>
+      <c r="A29" s="1" t="n">
+        <v>46255.75466435185</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1777,9 +1775,17 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K29" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
@@ -1788,13 +1794,13 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1804,104 +1810,96 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>46251.58453703704</v>
+      <c r="A30" s="1" t="n">
+        <v>46253.46241898148</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>736</v>
-      </c>
-      <c r="K30" t="n">
-        <v>736</v>
-      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>46245.37090277778</v>
+      <c r="A31" s="1" t="n">
+        <v>46251.58453703704</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K31" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
+      <c r="N31" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O31" s="1" t="n">
+        <v>46257</v>
+      </c>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
@@ -1912,113 +1910,125 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>46244.33856481482</v>
+      <c r="A32" s="1" t="n">
+        <v>46245.37090277778</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K32" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O32" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>46244.30862268519</v>
+      <c r="A33" s="1" t="n">
+        <v>46244.33856481482</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>785</v>
+      </c>
+      <c r="K33" t="n">
+        <v>785</v>
+      </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="N33" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O33" s="1" t="n">
+        <v>46251</v>
+      </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2028,68 +2038,56 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>46239.68305555556</v>
+      <c r="A34" s="1" t="n">
+        <v>46244.30862268519</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J34" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K34" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>46238.74310185185</v>
+      <c r="A35" s="1" t="n">
+        <v>46239.68305555556</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2099,9 +2097,17 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K35" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
@@ -2110,13 +2116,13 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2126,137 +2132,129 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>46234.89293981482</v>
+      <c r="A36" s="1" t="n">
+        <v>46238.74310185185</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J36" t="n">
-        <v>849</v>
-      </c>
-      <c r="K36" t="n">
-        <v>849</v>
-      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O36" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>46216.73908564815</v>
+      <c r="A37" s="1" t="n">
+        <v>46234.89293981482</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K37" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="N37" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O37" s="1" t="n">
+        <v>46243</v>
+      </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>46216.4634375</v>
+      <c r="A38" s="1" t="n">
+        <v>46216.73908564815</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2268,14 +2266,14 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K38" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
@@ -2285,13 +2283,13 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2301,125 +2299,121 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>46199</v>
-      </c>
+      <c r="A39" s="1" t="n">
+        <v>46216.4634375</v>
+      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M39" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N39" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K39" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B40" t="inlineStr"/>
+      <c r="A40" s="1" t="n">
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B40" s="1" t="n">
+        <v>46199</v>
+      </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K40" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M40" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N40" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O40" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2429,62 +2423,54 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>46146.4284375</v>
+      <c r="A41" s="1" t="n">
+        <v>46160.52664351852</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K41" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O41" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2494,58 +2480,62 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>46119.48518518519</v>
+      <c r="A42" s="1" t="n">
+        <v>46146.4284375</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K42" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="N42" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O42" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2555,38 +2545,38 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>46093.45828703704</v>
+      <c r="A43" s="1" t="n">
+        <v>46119.48518518519</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K43" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
@@ -2596,17 +2586,17 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2616,12 +2606,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B44" s="2" t="n">
-        <v>46070</v>
-      </c>
+      <c r="A44" s="1" t="n">
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
@@ -2630,48 +2618,46 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K44" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2681,26 +2667,26 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B45" s="2" t="n">
-        <v>46265</v>
+      <c r="A45" s="1" t="n">
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>46070</v>
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2711,30 +2697,32 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K45" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
+      <c r="N45" s="1" t="n">
+        <v>46068</v>
+      </c>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2744,155 +2732,153 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B46" t="inlineStr"/>
+      <c r="A46" s="1" t="n">
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>46265</v>
+      </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M46" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N46" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O46" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J46" t="n">
+        <v>603</v>
+      </c>
+      <c r="K46" t="n">
+        <v>603</v>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46062.51478009259</v>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0011-26</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M47" t="n">
+        <v>-90.10947400000001</v>
+      </c>
+      <c r="N47" s="1" t="n">
+        <v>46062</v>
+      </c>
+      <c r="O47" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
           <t>Amrize Dock on Mckellar Lake</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="S47" t="inlineStr">
         <is>
           <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="T47" t="inlineStr">
         <is>
           <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
         <v>46058.58436342593</v>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" s="2" t="n">
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0009-26</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>585</v>
-      </c>
-      <c r="K47" t="n">
-        <v>869</v>
-      </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr">
-        <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>46051.75101851852</v>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2908,15 +2894,15 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K48" t="n">
         <v>869</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" s="2" t="n">
-        <v>46052</v>
+      <c r="N48" s="1" t="n">
+        <v>46061</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
@@ -2926,14 +2912,14 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2943,12 +2929,12 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>46050.44465277778</v>
+      <c r="A49" s="1" t="n">
+        <v>46051.75101851852</v>
       </c>
       <c r="B49" t="inlineStr"/>
-      <c r="C49" s="2" t="n">
-        <v>46052</v>
+      <c r="C49" s="1" t="n">
+        <v>46061</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2957,7 +2943,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2976,17 +2962,17 @@
         <v>303</v>
       </c>
       <c r="K49" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" s="2" t="n">
-        <v>46050</v>
+      <c r="N49" s="1" t="n">
+        <v>46052</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -2998,7 +2984,7 @@
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -3008,12 +2994,12 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>46045.53974537037</v>
+      <c r="A50" s="1" t="n">
+        <v>46050.44465277778</v>
       </c>
       <c r="B50" t="inlineStr"/>
-      <c r="C50" s="2" t="n">
-        <v>46050</v>
+      <c r="C50" s="1" t="n">
+        <v>46052</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3022,7 +3008,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3045,8 +3031,8 @@
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" s="2" t="n">
-        <v>46045</v>
+      <c r="N50" s="1" t="n">
+        <v>46050</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
@@ -3063,137 +3049,141 @@
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" s="1" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>303</v>
+      </c>
+      <c r="K51" t="n">
+        <v>585</v>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" s="1" t="n">
+        <v>46045</v>
+      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
           <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
         <v>46042.81428240741</v>
-      </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0004-26</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M51" t="n">
-        <v>-90.10785143484679</v>
-      </c>
-      <c r="N51" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O51" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="T51" t="inlineStr">
-        <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
-        </is>
-      </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>46037.53365740741</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J52" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K52" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M52" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N52" s="1" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O52" s="1" t="n">
+        <v>46044</v>
+      </c>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -3203,26 +3193,24 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>46037.50987268519</v>
+      <c r="A53" s="1" t="n">
+        <v>46037.53365740741</v>
       </c>
       <c r="B53" t="inlineStr"/>
-      <c r="C53" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -3233,32 +3221,30 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K53" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3268,12 +3254,12 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>46033.86975694444</v>
+      <c r="A54" s="1" t="n">
+        <v>46037.50987268519</v>
       </c>
       <c r="B54" t="inlineStr"/>
-      <c r="C54" s="2" t="n">
-        <v>46037</v>
+      <c r="C54" s="1" t="n">
+        <v>46045</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3282,7 +3268,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3305,13 +3291,13 @@
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" s="2" t="n">
-        <v>46034</v>
+      <c r="N54" s="1" t="n">
+        <v>46037</v>
       </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -3323,10 +3309,75 @@
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>303</v>
+      </c>
+      <c r="K55" t="n">
+        <v>869</v>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="U55" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-23: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -417,126 +429,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U55"/>
+  <dimension ref="A1:U56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date_published</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cancelled_date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>replaced_date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>active?</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>message_id</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>other_notes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>dredge</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>river</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>mm_low</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>mm_high</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>lon</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>date_start</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>date_end</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>northbound</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>southbound</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>location_details</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>instructions</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>full_memo</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46286.49263888889</v>
+      <c r="A2" s="2" t="n">
+        <v>46288.45719907407</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0107-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,29 +567,25 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ON 22SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-42N 086-50-37W,30-23-16N 086-45-43W,30-22-02N 086-43-53W,30-11-30N 086-24-28W,30-09-46N 086-22-43W,30-05-13N 086-20-40W,29-59-57N 086-23-04W,29-53-34N 086-30-02W,29-53-39N 086-45-44W AND30-10-40N 086-46-44W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//221900Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>46283.70012731481</v>
+      <c r="A3" s="2" t="n">
+        <v>46286.49263888889</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0106-26</t>
+          <t>CGD-H BNM 0107-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -604,41 +612,33 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>ON 21SEP2026, 23SEP2026 AND 24SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-40N 086-50-41W,30-23-27N 086-44-14W,30-10-30N 086-36-30W,30-02-39N 086-36-05W,30-02-37N 086-46-12W AND30-10-45N 086-46-21W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//241300Z SEP 26// BT</t>
+          <t>ON 22SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-42N 086-50-37W,30-23-16N 086-45-43W,30-22-02N 086-43-53W,30-11-30N 086-24-28W,30-09-46N 086-22-43W,30-05-13N 086-20-40W,29-59-57N 086-23-04W,29-53-34N 086-30-02W,29-53-39N 086-45-44W AND30-10-40N 086-46-44W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//221900Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46283.699375</v>
+      <c r="A4" s="2" t="n">
+        <v>46283.70012731481</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
+          <t>CGD-H BNM 0106-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>587</v>
-      </c>
-      <c r="K4" t="n">
-        <v>593</v>
-      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -647,31 +647,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
+          <t>ON 21SEP2026, 23SEP2026 AND 24SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-40N 086-50-41W,30-23-27N 086-44-14W,30-10-30N 086-36-30W,30-02-39N 086-36-05W,30-02-37N 086-46-12W AND30-10-45N 086-46-21W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//241300Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46282.57303240741</v>
+      <c r="A5" s="2" t="n">
+        <v>46283.699375</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -680,52 +676,40 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>691</v>
+        <v>587</v>
       </c>
       <c r="K5" t="n">
-        <v>701.2</v>
+        <v>593</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" s="1" t="n">
-        <v>46277</v>
-      </c>
-      <c r="O5" s="1" t="n">
-        <v>46283</v>
-      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46281.77060185185</v>
+      <c r="A6" s="2" t="n">
+        <v>46282.57303240741</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
@@ -736,7 +720,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -747,7 +731,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Midway</t>
+          <t>Jadwin</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -756,30 +740,30 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>652</v>
+        <v>691</v>
       </c>
       <c r="K6" t="n">
-        <v>652</v>
+        <v>701.2</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" s="1" t="n">
-        <v>46281</v>
-      </c>
-      <c r="O6" s="1" t="n">
-        <v>46287</v>
+      <c r="N6" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>46283</v>
       </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Mariners are advised to transit the area with caution.</t>
+          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -789,88 +773,92 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46281.41737268519</v>
+      <c r="A7" s="2" t="n">
+        <v>46281.77060185185</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>652</v>
+      </c>
+      <c r="K7" t="n">
+        <v>652</v>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="N7" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>46287</v>
+      </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Mariners are advised to transit the area with caution.</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46280.38037037037</v>
+      <c r="A8" s="2" t="n">
+        <v>46281.41737268519</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>connected to above line</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>691</v>
-      </c>
-      <c r="K8" t="n">
-        <v>701</v>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
@@ -881,70 +869,68 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46278.72424768518</v>
+      <c r="A9" s="2" t="n">
+        <v>46280.38037037037</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>connected to above line</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>585</v>
+        <v>691</v>
       </c>
       <c r="K9" t="n">
-        <v>869</v>
+        <v>701</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" s="1" t="n">
-        <v>46278</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>11'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -954,7 +940,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>46278.72424768518</v>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -982,14 +968,14 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K10" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" s="1" t="n">
+      <c r="N10" s="2" t="n">
         <v>46278</v>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -1000,7 +986,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>12'6" draft. 7 barges wide.</t>
+          <t>11'6" draft. 7 barges wide.</t>
         </is>
       </c>
       <c r="R10" t="inlineStr"/>
@@ -1017,8 +1003,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>46277.53633101852</v>
+      <c r="A11" s="2" t="n">
+        <v>46278.72424768518</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
@@ -1029,12 +1015,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1045,22 +1031,32 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>482</v>
+        <v>303</v>
       </c>
       <c r="K11" t="n">
-        <v>482</v>
+        <v>585</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>12'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1070,27 +1066,39 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>46277.09849537037</v>
+      <c r="A12" s="2" t="n">
+        <v>46277.53633101852</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>482</v>
+      </c>
+      <c r="K12" t="n">
+        <v>482</v>
+      </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -1101,41 +1109,37 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr"/>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>46276.67863425926</v>
+      <c r="A13" s="2" t="n">
+        <v>46277.09849537037</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>303</v>
-      </c>
-      <c r="K13" t="n">
-        <v>869</v>
-      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1146,111 +1150,115 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>46275.97677083333</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>46291</v>
-      </c>
+      <c r="A14" s="2" t="n">
+        <v>46276.67863425926</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K14" t="n">
-        <v>663</v>
+        <v>869</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" s="1" t="n">
-        <v>46275</v>
-      </c>
-      <c r="O14" s="1" t="n">
-        <v>46281</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>n</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>46273.435</v>
-      </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="A15" s="2" t="n">
+        <v>46275.97677083333</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46291</v>
+      </c>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>663</v>
+      </c>
+      <c r="K15" t="n">
+        <v>663</v>
+      </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="N15" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>46281</v>
+      </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1260,39 +1268,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>46268.97141203703</v>
+      <c r="A16" s="2" t="n">
+        <v>46273.435</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>303</v>
-      </c>
-      <c r="K16" t="n">
-        <v>869</v>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1303,37 +1299,49 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>46268.53527777778</v>
+      <c r="A17" s="2" t="n">
+        <v>46268.97141203703</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>303</v>
+      </c>
+      <c r="K17" t="n">
+        <v>869</v>
+      </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
@@ -1344,21 +1352,25 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr"/>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>46265.53005787037</v>
+      <c r="A18" s="2" t="n">
+        <v>46268.53527777778</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1381,14 +1393,14 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>46265.52835648148</v>
+      <c r="A19" s="2" t="n">
+        <v>46265.53005787037</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -1418,21 +1430,21 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>46265.52792824074</v>
+      <c r="A20" s="2" t="n">
+        <v>46265.52835648148</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1455,21 +1467,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>46265.52664351852</v>
+      <c r="A21" s="2" t="n">
+        <v>46265.52792824074</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1492,21 +1504,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>46265.52623842593</v>
+      <c r="A22" s="2" t="n">
+        <v>46265.52664351852</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1529,21 +1541,21 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>46265.52559027778</v>
+      <c r="A23" s="2" t="n">
+        <v>46265.52623842593</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1566,21 +1578,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>46265.52508101852</v>
+      <c r="A24" s="2" t="n">
+        <v>46265.52559027778</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1603,21 +1615,21 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>46265.52371527778</v>
+      <c r="A25" s="2" t="n">
+        <v>46265.52508101852</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1640,21 +1652,21 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>46258.44554398148</v>
+      <c r="A26" s="2" t="n">
+        <v>46265.52371527778</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1677,21 +1689,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>46258.44363425926</v>
+      <c r="A27" s="2" t="n">
+        <v>46258.44554398148</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1714,21 +1726,21 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>46257.8184375</v>
+      <c r="A28" s="2" t="n">
+        <v>46258.44363425926</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1751,21 +1763,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>46255.75466435185</v>
+      <c r="A29" s="2" t="n">
+        <v>46257.8184375</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1775,50 +1787,34 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K29" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>46253.46241898148</v>
+      <c r="A30" s="2" t="n">
+        <v>46255.75466435185</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1828,9 +1824,17 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K30" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
@@ -1839,13 +1843,13 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1855,104 +1859,96 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>46251.58453703704</v>
+      <c r="A31" s="2" t="n">
+        <v>46253.46241898148</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>736</v>
-      </c>
-      <c r="K31" t="n">
-        <v>736</v>
-      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" s="1" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O31" s="1" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
-        <v>46245.37090277778</v>
+      <c r="A32" s="2" t="n">
+        <v>46251.58453703704</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K32" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
@@ -1963,113 +1959,125 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>46244.33856481482</v>
+      <c r="A33" s="2" t="n">
+        <v>46245.37090277778</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K33" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" s="1" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O33" s="1" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>46244.30862268519</v>
+      <c r="A34" s="2" t="n">
+        <v>46244.33856481482</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>785</v>
+      </c>
+      <c r="K34" t="n">
+        <v>785</v>
+      </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+      <c r="N34" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2079,68 +2087,56 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>46239.68305555556</v>
+      <c r="A35" s="2" t="n">
+        <v>46244.30862268519</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J35" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K35" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>46238.74310185185</v>
+      <c r="A36" s="2" t="n">
+        <v>46239.68305555556</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2150,9 +2146,17 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K36" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
@@ -2161,13 +2165,13 @@
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2177,137 +2181,129 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>46234.89293981482</v>
+      <c r="A37" s="2" t="n">
+        <v>46238.74310185185</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>849</v>
-      </c>
-      <c r="K37" t="n">
-        <v>849</v>
-      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" s="1" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O37" s="1" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>46216.73908564815</v>
+      <c r="A38" s="2" t="n">
+        <v>46234.89293981482</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K38" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="N38" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>46216.4634375</v>
+      <c r="A39" s="2" t="n">
+        <v>46216.73908564815</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2319,14 +2315,14 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K39" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
@@ -2336,13 +2332,13 @@
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2352,125 +2348,121 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B40" s="1" t="n">
-        <v>46199</v>
-      </c>
+      <c r="A40" s="2" t="n">
+        <v>46216.4634375</v>
+      </c>
+      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N40" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O40" s="1" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K40" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B41" t="inlineStr"/>
+      <c r="A41" s="2" t="n">
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K41" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M41" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2480,62 +2472,54 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>46146.4284375</v>
+      <c r="A42" s="2" t="n">
+        <v>46160.52664351852</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K42" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O42" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2545,58 +2529,62 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>46119.48518518519</v>
+      <c r="A43" s="2" t="n">
+        <v>46146.4284375</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K43" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="N43" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2606,38 +2594,38 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>46093.45828703704</v>
+      <c r="A44" s="2" t="n">
+        <v>46119.48518518519</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K44" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
@@ -2647,17 +2635,17 @@
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2667,12 +2655,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B45" s="1" t="n">
-        <v>46070</v>
-      </c>
+      <c r="A45" s="2" t="n">
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
@@ -2681,48 +2667,46 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K45" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2732,26 +2716,26 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B46" s="1" t="n">
-        <v>46265</v>
+      <c r="A46" s="2" t="n">
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>46070</v>
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -2762,30 +2746,32 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K46" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="N46" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2795,155 +2781,153 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B47" t="inlineStr"/>
+      <c r="A47" s="2" t="n">
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>46265</v>
+      </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M47" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N47" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O47" s="1" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J47" t="n">
+        <v>603</v>
+      </c>
+      <c r="K47" t="n">
+        <v>603</v>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46062.51478009259</v>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0011-26</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M48" t="n">
+        <v>-90.10947400000001</v>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
           <t>Amrize Dock on Mckellar Lake</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr">
+      <c r="S48" t="inlineStr">
         <is>
           <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
-      <c r="T47" t="inlineStr">
+      <c r="T48" t="inlineStr">
         <is>
           <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
         <v>46058.58436342593</v>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" s="1" t="n">
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" s="2" t="n">
         <v>46068</v>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0009-26</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>585</v>
-      </c>
-      <c r="K48" t="n">
-        <v>869</v>
-      </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr">
-        <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>46051.75101851852</v>
-      </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2959,15 +2943,15 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K49" t="n">
         <v>869</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" s="1" t="n">
-        <v>46052</v>
+      <c r="N49" s="2" t="n">
+        <v>46061</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
@@ -2977,14 +2961,14 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2994,12 +2978,12 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>46050.44465277778</v>
+      <c r="A50" s="2" t="n">
+        <v>46051.75101851852</v>
       </c>
       <c r="B50" t="inlineStr"/>
-      <c r="C50" s="1" t="n">
-        <v>46052</v>
+      <c r="C50" s="2" t="n">
+        <v>46061</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3008,7 +2992,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3027,17 +3011,17 @@
         <v>303</v>
       </c>
       <c r="K50" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" s="1" t="n">
-        <v>46050</v>
+      <c r="N50" s="2" t="n">
+        <v>46052</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -3049,7 +3033,7 @@
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -3059,12 +3043,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>46045.53974537037</v>
+      <c r="A51" s="2" t="n">
+        <v>46050.44465277778</v>
       </c>
       <c r="B51" t="inlineStr"/>
-      <c r="C51" s="1" t="n">
-        <v>46050</v>
+      <c r="C51" s="2" t="n">
+        <v>46052</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3073,7 +3057,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3096,8 +3080,8 @@
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
-      <c r="N51" s="1" t="n">
-        <v>46045</v>
+      <c r="N51" s="2" t="n">
+        <v>46050</v>
       </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
@@ -3114,137 +3098,141 @@
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>303</v>
+      </c>
+      <c r="K52" t="n">
+        <v>585</v>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
+        <is>
           <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
         <v>46042.81428240741</v>
-      </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0004-26</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M52" t="n">
-        <v>-90.10785143484679</v>
-      </c>
-      <c r="N52" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O52" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
-        </is>
-      </c>
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>46037.53365740741</v>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J53" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K53" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M53" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3254,26 +3242,24 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>46037.50987268519</v>
+      <c r="A54" s="2" t="n">
+        <v>46037.53365740741</v>
       </c>
       <c r="B54" t="inlineStr"/>
-      <c r="C54" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
@@ -3284,32 +3270,30 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K54" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3319,12 +3303,12 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>46033.86975694444</v>
+      <c r="A55" s="2" t="n">
+        <v>46037.50987268519</v>
       </c>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" s="1" t="n">
-        <v>46037</v>
+      <c r="C55" s="2" t="n">
+        <v>46045</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3333,7 +3317,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3356,13 +3340,13 @@
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" s="1" t="n">
-        <v>46034</v>
+      <c r="N55" s="2" t="n">
+        <v>46037</v>
       </c>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -3374,10 +3358,75 @@
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>303</v>
+      </c>
+      <c r="K56" t="n">
+        <v>869</v>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="U56" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-24: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U56"/>
+  <dimension ref="A1:U57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46288.45719907407</v>
+        <v>46288.66804398148</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -571,21 +571,21 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
+          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46286.49263888889</v>
+        <v>46288.45719907407</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0107-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -604,29 +604,25 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>ON 22SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-42N 086-50-37W,30-23-16N 086-45-43W,30-22-02N 086-43-53W,30-11-30N 086-24-28W,30-09-46N 086-22-43W,30-05-13N 086-20-40W,29-59-57N 086-23-04W,29-53-34N 086-30-02W,29-53-39N 086-45-44W AND30-10-40N 086-46-44W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//221900Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46283.70012731481</v>
+        <v>46286.49263888889</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0106-26</t>
+          <t>CGD-H BNM 0107-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -653,41 +649,33 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>ON 21SEP2026, 23SEP2026 AND 24SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-40N 086-50-41W,30-23-27N 086-44-14W,30-10-30N 086-36-30W,30-02-39N 086-36-05W,30-02-37N 086-46-12W AND30-10-45N 086-46-21W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//241300Z SEP 26// BT</t>
+          <t>ON 22SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-42N 086-50-37W,30-23-16N 086-45-43W,30-22-02N 086-43-53W,30-11-30N 086-24-28W,30-09-46N 086-22-43W,30-05-13N 086-20-40W,29-59-57N 086-23-04W,29-53-34N 086-30-02W,29-53-39N 086-45-44W AND30-10-40N 086-46-44W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//221900Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46283.699375</v>
+        <v>46283.70012731481</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
+          <t>CGD-H BNM 0106-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>587</v>
-      </c>
-      <c r="K5" t="n">
-        <v>593</v>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -696,31 +684,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
+          <t>ON 21SEP2026, 23SEP2026 AND 24SEP2026, FROM 1200Z TO 1800Z, THE U.S. AIR FORCE WILL CONDUCT TESTING OPERATIONS OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-22-40N 086-50-41W,30-23-27N 086-44-14W,30-10-30N 086-36-30W,30-02-39N 086-36-05W,30-02-37N 086-46-12W AND30-10-45N 086-46-21W.MARINERS SHOULD AVOID THE HAZARD AREA DURING THE TESTS.CANCEL AT//241300Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46282.57303240741</v>
+        <v>46283.699375</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -729,52 +713,40 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>691</v>
+        <v>587</v>
       </c>
       <c r="K6" t="n">
-        <v>701.2</v>
+        <v>593</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" s="2" t="n">
-        <v>46277</v>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>46283</v>
-      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46281.77060185185</v>
+        <v>46282.57303240741</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
@@ -785,7 +757,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -796,7 +768,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Midway</t>
+          <t>Jadwin</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -805,30 +777,30 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>652</v>
+        <v>691</v>
       </c>
       <c r="K7" t="n">
-        <v>652</v>
+        <v>701.2</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>46281</v>
+        <v>46277</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>46287</v>
+        <v>46283</v>
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Mariners are advised to transit the area with caution.</t>
+          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -839,87 +811,91 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46281.41737268519</v>
+        <v>46281.77060185185</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>652</v>
+      </c>
+      <c r="K8" t="n">
+        <v>652</v>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="N8" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>46287</v>
+      </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Mariners are advised to transit the area with caution.</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>connected to above line</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>691</v>
-      </c>
-      <c r="K9" t="n">
-        <v>701</v>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -930,70 +906,68 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>connected to above line</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>585</v>
+        <v>691</v>
       </c>
       <c r="K10" t="n">
-        <v>869</v>
+        <v>701</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" s="2" t="n">
-        <v>46278</v>
-      </c>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>11'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1031,10 +1005,10 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K11" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
@@ -1049,7 +1023,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>12'6" draft. 7 barges wide.</t>
+          <t>11'6" draft. 7 barges wide.</t>
         </is>
       </c>
       <c r="R11" t="inlineStr"/>
@@ -1067,7 +1041,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
@@ -1078,12 +1052,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1094,22 +1068,32 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>482</v>
+        <v>303</v>
       </c>
       <c r="K12" t="n">
-        <v>482</v>
+        <v>585</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>12'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1120,26 +1104,38 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>482</v>
+      </c>
+      <c r="K13" t="n">
+        <v>482</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1150,41 +1146,37 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr"/>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>303</v>
-      </c>
-      <c r="K14" t="n">
-        <v>869</v>
-      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
@@ -1195,111 +1187,115 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46275.97677083333</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>46291</v>
-      </c>
+        <v>46276.67863425926</v>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K15" t="n">
-        <v>663</v>
+        <v>869</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>46281</v>
-      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>n</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46273.435</v>
-      </c>
-      <c r="B16" t="inlineStr"/>
+        <v>46275.97677083333</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46291</v>
+      </c>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>663</v>
+      </c>
+      <c r="K16" t="n">
+        <v>663</v>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="N16" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>46281</v>
+      </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1310,38 +1306,26 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46273.435</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>303</v>
-      </c>
-      <c r="K17" t="n">
-        <v>869</v>
-      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
@@ -1352,37 +1336,49 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>303</v>
+      </c>
+      <c r="K18" t="n">
+        <v>869</v>
+      </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
@@ -1393,21 +1389,25 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr"/>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1430,14 +1430,14 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
@@ -1467,21 +1467,21 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1504,21 +1504,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1541,21 +1541,21 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1578,21 +1578,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1615,21 +1615,21 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1652,21 +1652,21 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1689,21 +1689,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1726,21 +1726,21 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1763,21 +1763,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1800,21 +1800,21 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1824,50 +1824,34 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K30" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1877,9 +1861,17 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K31" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
@@ -1888,13 +1880,13 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1905,103 +1897,95 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J32" t="n">
-        <v>736</v>
-      </c>
-      <c r="K32" t="n">
-        <v>736</v>
-      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O32" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K33" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="N33" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
@@ -2012,113 +1996,125 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K34" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O34" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>785</v>
+      </c>
+      <c r="K35" t="n">
+        <v>785</v>
+      </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
+      <c r="N35" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2129,67 +2125,55 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J36" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K36" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2199,9 +2183,17 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K37" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
@@ -2210,13 +2202,13 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2227,136 +2219,128 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>849</v>
-      </c>
-      <c r="K38" t="n">
-        <v>849</v>
-      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O38" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K39" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="N39" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2368,14 +2352,14 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K40" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
@@ -2385,13 +2369,13 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2402,124 +2386,120 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B41" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M41" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N41" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O41" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K41" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B42" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K42" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M42" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2530,61 +2510,53 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K43" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O43" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2595,57 +2567,61 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K44" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="N44" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2656,37 +2632,37 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K45" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
@@ -2696,17 +2672,17 @@
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2717,11 +2693,9 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B46" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
@@ -2730,48 +2704,46 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K46" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2782,25 +2754,25 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46065.67140046296</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>46265</v>
+        <v>46070</v>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2811,30 +2783,32 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K47" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
+      <c r="N47" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2845,65 +2819,59 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B48" t="inlineStr"/>
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>46265</v>
+      </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M48" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N48" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O48" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J48" t="n">
+        <v>603</v>
+      </c>
+      <c r="K48" t="n">
+        <v>603</v>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2914,12 +2882,10 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B49" t="inlineStr"/>
-      <c r="C49" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>N</t>
@@ -2927,48 +2893,54 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>585</v>
-      </c>
-      <c r="K49" t="n">
-        <v>869</v>
-      </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M49" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N49" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O49" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2979,11 +2951,11 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2992,7 +2964,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3008,7 +2980,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K50" t="n">
         <v>869</v>
@@ -3016,7 +2988,7 @@
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
@@ -3026,14 +2998,14 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -3044,11 +3016,11 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3057,7 +3029,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3076,17 +3048,17 @@
         <v>303</v>
       </c>
       <c r="K51" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -3098,7 +3070,7 @@
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -3109,11 +3081,11 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -3122,7 +3094,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3146,7 +3118,7 @@
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
@@ -3163,7 +3135,7 @@
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -3174,10 +3146,12 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>N</t>
@@ -3185,54 +3159,48 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M53" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J53" t="n">
+        <v>303</v>
+      </c>
+      <c r="K53" t="n">
+        <v>585</v>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
       <c r="N53" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O53" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3243,57 +3211,65 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J54" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K54" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M54" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3304,25 +3280,23 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -3333,32 +3307,30 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K55" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3369,11 +3341,11 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3382,7 +3354,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3406,12 +3378,12 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -3423,10 +3395,75 @@
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>303</v>
+      </c>
+      <c r="K57" t="n">
+        <v>869</v>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="U57" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-30: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -1242,10 +1242,10 @@
         </is>
       </c>
       <c r="J16" t="n">
+        <v>303</v>
+      </c>
+      <c r="K16" t="n">
         <v>585</v>
-      </c>
-      <c r="K16" t="n">
-        <v>869</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>11'6" draft. 7 barges wide.</t>
+          <t>12'6" draft. 7 barges wide.</t>
         </is>
       </c>
       <c r="R16" t="inlineStr"/>
@@ -1305,10 +1305,10 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K17" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>12'6" draft. 7 barges wide.</t>
+          <t>11'6" draft. 7 barges wide.</t>
         </is>
       </c>
       <c r="R17" t="inlineStr"/>

</xml_diff>

<commit_message>
Daily pipeline 2026-10-01: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U62"/>
+  <dimension ref="A1:U63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294.51650462963</v>
+        <v>46296.38649305556</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0110-26</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -567,49 +567,37 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-35-28.92N 095-50-49.62W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//060500Z OCT 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46293.87546296296</v>
+        <v>46294.51650462963</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>CGD-H BNM 0110-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>408</v>
-      </c>
-      <c r="K3" t="n">
-        <v>486.2</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,64 +606,76 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-35-28.92N 095-50-49.62W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//060500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46293.58675925926</v>
+        <v>46293.87546296296</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0108-26</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>408</v>
+      </c>
+      <c r="K4" t="n">
+        <v>486.2</v>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0108-26 DTG 251747Z SEP 262. STARSHIP FLIGHT 14 MISSION COMPLETE. BT</t>
+          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46293.48982638889</v>
+        <v>46293.58675925926</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0109-26</t>
+          <t>CGD-H BNM 0108-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -694,29 +694,25 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-31-21.06N 095-56-45.54W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//050500Z OCT 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0108-26 DTG 251747Z SEP 262. STARSHIP FLIGHT 14 MISSION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46293.48231481481</v>
+        <v>46293.48982638889</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>CGD-H BNM 0109-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -735,25 +731,29 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-31-21.06N 095-56-45.54W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//050500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46290.60001157408</v>
+        <v>46293.48231481481</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0108-26</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -772,49 +772,37 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
-        </is>
-      </c>
+      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 14:A. HIGH RISK HAZARD AREA25-12-00N 092-58-00W,25-31-00N 093-52-00W,25-42-00N 095-24-00W,26-02-00N 096-32-00W,26-04-00N 096-49-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-41-00N 096-47-00W,25-02-00N 095-05-00W,24-29-00N 094-08-00W,24-20-00N 093-32-00W,24-25-00N 092-52-00W AND24-45-00N 092-43-00W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-04-00N 096-49-00W,26-01-00N 096-17-00W,26-01-00N 095-12-00W,25-59-00N 094-36-00W,25-59-00N 094-05-00W,25-25-00N 093-06-00W,25-31-00N 091-46-00W,23-32-00N 088-52-00W,23-04-00N 088-33-00W,22-03-00N 086-24-00W,21-38-00N 084-59-00W,20-59-00N 082-38-00W,20-43-00N 081-42-00W,20-07-00N 079-44-00W,19-46-00N 078-47-00W,19-23-00N 078-04-00W,19-19-00N 078-18-00W,19-34-00N 079-19-00W,19-44-00N 079-44-00W,20-12-00N 081-13-00W,20-43-00N 083-13-00W,21-06-00N 084-54-00W,21-43-00N 086-42-00W,21-59-00N 087-26-00W,22-39-00N 089-10-00W,22-45-00N 089-41-00W,22-58-00N 092-36-00W,24-18-00N 095-02-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:28/1215Z SEP 26 TO 28/1414Z SEP 2629/1215Z SEP 26 TO 29/1414Z SEP 2630/1215Z SEP 26 TO 30/1414Z SEP 2601/1215Z OCT 26 TO 01/1414Z OCT 2602/1215Z OCT 26 TO 02/1414Z OCT 2603/1215Z OCT 26 TO 03/1414Z OCT 2604/1215Z OCT 26 TO 04/1414Z OCT 263. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//041514Z OCT 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46290.59799768519</v>
+        <v>46290.60001157408</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>CGD-H BNM 0108-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>481</v>
-      </c>
-      <c r="K8" t="n">
-        <v>484</v>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
@@ -823,68 +811,76 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 14:A. HIGH RISK HAZARD AREA25-12-00N 092-58-00W,25-31-00N 093-52-00W,25-42-00N 095-24-00W,26-02-00N 096-32-00W,26-04-00N 096-49-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-41-00N 096-47-00W,25-02-00N 095-05-00W,24-29-00N 094-08-00W,24-20-00N 093-32-00W,24-25-00N 092-52-00W AND24-45-00N 092-43-00W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-04-00N 096-49-00W,26-01-00N 096-17-00W,26-01-00N 095-12-00W,25-59-00N 094-36-00W,25-59-00N 094-05-00W,25-25-00N 093-06-00W,25-31-00N 091-46-00W,23-32-00N 088-52-00W,23-04-00N 088-33-00W,22-03-00N 086-24-00W,21-38-00N 084-59-00W,20-59-00N 082-38-00W,20-43-00N 081-42-00W,20-07-00N 079-44-00W,19-46-00N 078-47-00W,19-23-00N 078-04-00W,19-19-00N 078-18-00W,19-34-00N 079-19-00W,19-44-00N 079-44-00W,20-12-00N 081-13-00W,20-43-00N 083-13-00W,21-06-00N 084-54-00W,21-43-00N 086-42-00W,21-59-00N 087-26-00W,22-39-00N 089-10-00W,22-45-00N 089-41-00W,22-58-00N 092-36-00W,24-18-00N 095-02-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:28/1215Z SEP 26 TO 28/1414Z SEP 2629/1215Z SEP 26 TO 29/1414Z SEP 2630/1215Z SEP 26 TO 30/1414Z SEP 2601/1215Z OCT 26 TO 01/1414Z OCT 2602/1215Z OCT 26 TO 02/1414Z OCT 2603/1215Z OCT 26 TO 03/1414Z OCT 2604/1215Z OCT 26 TO 04/1414Z OCT 263. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//041514Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46288.66804398148</v>
+        <v>46290.59799768519</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>481</v>
+      </c>
+      <c r="K9" t="n">
+        <v>484</v>
+      </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46288.45719907407</v>
+        <v>46288.66804398148</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -907,7 +903,7 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
+          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -918,72 +914,48 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46283.699375</v>
+        <v>46288.45719907407</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>587</v>
-      </c>
-      <c r="K11" t="n">
-        <v>593</v>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" s="2" t="n">
-        <v>46284</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>46285</v>
-      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>Cumbyville</t>
-        </is>
-      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46282.57303240741</v>
+        <v>46283.699375</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
@@ -994,7 +966,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1014,30 +986,30 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>691</v>
+        <v>587</v>
       </c>
       <c r="K12" t="n">
-        <v>701.2</v>
+        <v>593</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>46277</v>
+        <v>46284</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>46283</v>
+        <v>46285</v>
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Cumbyville</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1048,7 +1020,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46281.77060185185</v>
+        <v>46282.57303240741</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
@@ -1059,7 +1031,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1070,7 +1042,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Midway</t>
+          <t>Jadwin</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1079,30 +1051,30 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>652</v>
+        <v>691</v>
       </c>
       <c r="K13" t="n">
-        <v>652</v>
+        <v>701.2</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>46281</v>
+        <v>46277</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>46287</v>
+        <v>46283</v>
       </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Mariners are advised to transit the area with caution.</t>
+          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1113,87 +1085,91 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46281.41737268519</v>
+        <v>46281.77060185185</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>652</v>
+      </c>
+      <c r="K14" t="n">
+        <v>652</v>
+      </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="N14" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>46287</v>
+      </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Mariners are advised to transit the area with caution.</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>connected to above line</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>691</v>
-      </c>
-      <c r="K15" t="n">
-        <v>701</v>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
@@ -1204,70 +1180,68 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>connected to above line</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>303</v>
+        <v>691</v>
       </c>
       <c r="K16" t="n">
-        <v>585</v>
+        <v>701</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" s="2" t="n">
-        <v>46278</v>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>12'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1305,10 +1279,10 @@
         </is>
       </c>
       <c r="J17" t="n">
+        <v>303</v>
+      </c>
+      <c r="K17" t="n">
         <v>585</v>
-      </c>
-      <c r="K17" t="n">
-        <v>869</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
@@ -1323,7 +1297,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>11'6" draft. 7 barges wide.</t>
+          <t>12'6" draft. 7 barges wide.</t>
         </is>
       </c>
       <c r="R17" t="inlineStr"/>
@@ -1341,7 +1315,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -1352,12 +1326,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1368,22 +1342,32 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>482</v>
+        <v>585</v>
       </c>
       <c r="K18" t="n">
-        <v>482</v>
+        <v>869</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>11'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1394,26 +1378,38 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>482</v>
+      </c>
+      <c r="K19" t="n">
+        <v>482</v>
+      </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
@@ -1424,41 +1420,37 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr"/>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>303</v>
-      </c>
-      <c r="K20" t="n">
-        <v>869</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
@@ -1469,111 +1461,115 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46275.97677083333</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>46291</v>
-      </c>
+        <v>46276.67863425926</v>
+      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K21" t="n">
-        <v>663</v>
+        <v>869</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="O21" s="2" t="n">
-        <v>46281</v>
-      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>n</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46273.435</v>
-      </c>
-      <c r="B22" t="inlineStr"/>
+        <v>46275.97677083333</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>46291</v>
+      </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>663</v>
+      </c>
+      <c r="K22" t="n">
+        <v>663</v>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="N22" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>46281</v>
+      </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1584,38 +1580,26 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46273.435</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>303</v>
-      </c>
-      <c r="K23" t="n">
-        <v>869</v>
-      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
@@ -1626,37 +1610,49 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>303</v>
+      </c>
+      <c r="K24" t="n">
+        <v>869</v>
+      </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
@@ -1667,21 +1663,25 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1704,14 +1704,14 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
@@ -1741,21 +1741,21 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1778,21 +1778,21 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1815,21 +1815,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1852,21 +1852,21 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1889,21 +1889,21 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1926,21 +1926,21 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1963,21 +1963,21 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2000,21 +2000,21 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2037,21 +2037,21 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2074,21 +2074,21 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2098,50 +2098,34 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J36" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K36" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2151,9 +2135,17 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K37" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
@@ -2162,13 +2154,13 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2179,103 +2171,95 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>736</v>
-      </c>
-      <c r="K38" t="n">
-        <v>736</v>
-      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O38" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K39" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="N39" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
@@ -2286,113 +2270,125 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K40" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>785</v>
+      </c>
+      <c r="K41" t="n">
+        <v>785</v>
+      </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="N41" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2403,67 +2399,55 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K42" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2473,9 +2457,17 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K43" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
@@ -2484,13 +2476,13 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2501,136 +2493,128 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J44" t="n">
-        <v>849</v>
-      </c>
-      <c r="K44" t="n">
-        <v>849</v>
-      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O44" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K45" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
+      <c r="N45" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2642,14 +2626,14 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K46" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
@@ -2659,13 +2643,13 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2676,124 +2660,120 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B47" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M47" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N47" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O47" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K47" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B48" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K48" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M48" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2804,61 +2784,53 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J49" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K49" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O49" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2869,57 +2841,61 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K50" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="N50" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2930,37 +2906,37 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K51" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
@@ -2970,17 +2946,17 @@
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2991,11 +2967,9 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B52" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
@@ -3004,48 +2978,46 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K52" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -3056,25 +3028,25 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46065.67140046296</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>46265</v>
+        <v>46070</v>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -3085,30 +3057,32 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K53" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3119,65 +3093,59 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B54" t="inlineStr"/>
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>46265</v>
+      </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M54" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N54" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O54" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J54" t="n">
+        <v>603</v>
+      </c>
+      <c r="K54" t="n">
+        <v>603</v>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3188,12 +3156,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>N</t>
@@ -3201,48 +3167,54 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J55" t="n">
-        <v>585</v>
-      </c>
-      <c r="K55" t="n">
-        <v>869</v>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M55" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N55" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3253,11 +3225,11 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3266,7 +3238,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3282,7 +3254,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K56" t="n">
         <v>869</v>
@@ -3290,7 +3262,7 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
@@ -3300,14 +3272,14 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3318,11 +3290,11 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -3331,7 +3303,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3350,17 +3322,17 @@
         <v>303</v>
       </c>
       <c r="K57" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
       <c r="N57" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -3372,7 +3344,7 @@
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -3383,11 +3355,11 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3396,7 +3368,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3420,7 +3392,7 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
       <c r="N58" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
@@ -3437,7 +3409,7 @@
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -3448,10 +3420,12 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>N</t>
@@ -3459,54 +3433,48 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M59" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J59" t="n">
+        <v>303</v>
+      </c>
+      <c r="K59" t="n">
+        <v>585</v>
+      </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
       <c r="N59" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O59" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S59" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -3517,57 +3485,65 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J60" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K60" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M60" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -3578,25 +3554,23 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -3607,32 +3581,30 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K61" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q61" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -3643,11 +3615,11 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3656,7 +3628,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3680,12 +3652,12 @@
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
       <c r="N62" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -3697,10 +3669,75 @@
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>303</v>
+      </c>
+      <c r="K63" t="n">
+        <v>869</v>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="U63" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-10-02: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U63"/>
+  <dimension ref="A1:U66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46296.38649305556</v>
+        <v>46297.52145833334</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>CGD-H BNM 0111-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -567,25 +567,29 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>MS - LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
+          <t>AUTONOMOUS SURFACE VESSEL (ASV) OPERATIONS ARE TAKINGPLACE BY THE ASV SEA ARCHER IN THE GULF OF AMERICA IN AN AREA BOUND BY APPROXIMATE POSITIONS:30-01-49N 088-44-36W,30-01-49N 088-13-25W,29-34-49N 088-13-25W AND29-34-49N 088-44-28W.MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE VESSELS.CANCEL AT//310500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46294.51650462963</v>
+        <v>46296.58851851852</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0110-26</t>
+          <t>SEC LMR BNM 0063-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -595,9 +599,17 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="K3" t="n">
+        <v>40.8</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -606,32 +618,32 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-35-28.92N 095-50-49.62W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//060500Z OCT 26// BT</t>
+          <t>1. MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ARE OUT ON THE JONESVILLE BRIDGE, MM 40.8 OUACHITA/BLACK RIVER.2. ALL MARINERS ARE REQUESTED TO TRANSIT WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46293.87546296296</v>
+        <v>46296.58818287037</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>SEC LMR BNM 0064-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -642,10 +654,10 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>408</v>
+        <v>57.3</v>
       </c>
       <c r="K4" t="n">
-        <v>486.2</v>
+        <v>57.3</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
@@ -655,27 +667,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
+          <t>1. MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ARE OUT ON THE HARRISONBURG BRIDGE, MM 57.3 OUACHITA/BLACK RIVER.2. ALL MARINERS ARE REQUESTED TO TRANSIT WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46293.58675925926</v>
+        <v>46296.38649305556</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0108-26</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -698,21 +710,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0108-26 DTG 251747Z SEP 262. STARSHIP FLIGHT 14 MISSION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46293.48982638889</v>
+        <v>46294.51650462963</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0109-26</t>
+          <t>CGD-H BNM 0110-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -739,51 +751,63 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-31-21.06N 095-56-45.54W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//050500Z OCT 26// BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-35-28.92N 095-50-49.62W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//060500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46293.48231481481</v>
+        <v>46293.87546296296</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>408</v>
+      </c>
+      <c r="K7" t="n">
+        <v>486.2</v>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46290.60001157408</v>
+        <v>46293.58675925926</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
@@ -809,49 +833,37 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 14:A. HIGH RISK HAZARD AREA25-12-00N 092-58-00W,25-31-00N 093-52-00W,25-42-00N 095-24-00W,26-02-00N 096-32-00W,26-04-00N 096-49-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-41-00N 096-47-00W,25-02-00N 095-05-00W,24-29-00N 094-08-00W,24-20-00N 093-32-00W,24-25-00N 092-52-00W AND24-45-00N 092-43-00W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-04-00N 096-49-00W,26-01-00N 096-17-00W,26-01-00N 095-12-00W,25-59-00N 094-36-00W,25-59-00N 094-05-00W,25-25-00N 093-06-00W,25-31-00N 091-46-00W,23-32-00N 088-52-00W,23-04-00N 088-33-00W,22-03-00N 086-24-00W,21-38-00N 084-59-00W,20-59-00N 082-38-00W,20-43-00N 081-42-00W,20-07-00N 079-44-00W,19-46-00N 078-47-00W,19-23-00N 078-04-00W,19-19-00N 078-18-00W,19-34-00N 079-19-00W,19-44-00N 079-44-00W,20-12-00N 081-13-00W,20-43-00N 083-13-00W,21-06-00N 084-54-00W,21-43-00N 086-42-00W,21-59-00N 087-26-00W,22-39-00N 089-10-00W,22-45-00N 089-41-00W,22-58-00N 092-36-00W,24-18-00N 095-02-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:28/1215Z SEP 26 TO 28/1414Z SEP 2629/1215Z SEP 26 TO 29/1414Z SEP 2630/1215Z SEP 26 TO 30/1414Z SEP 2601/1215Z OCT 26 TO 01/1414Z OCT 2602/1215Z OCT 26 TO 02/1414Z OCT 2603/1215Z OCT 26 TO 03/1414Z OCT 2604/1215Z OCT 26 TO 04/1414Z OCT 263. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//041514Z OCT 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0108-26 DTG 251747Z SEP 262. STARSHIP FLIGHT 14 MISSION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46290.59799768519</v>
+        <v>46293.48982638889</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>CGD-H BNM 0109-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>481</v>
-      </c>
-      <c r="K9" t="n">
-        <v>484</v>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -860,27 +872,27 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 27-31-21.06N 095-56-45.54W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//050500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46288.66804398148</v>
+        <v>46293.48231481481</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -903,25 +915,21 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46288.45719907407</v>
+        <v>46290.60001157408</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>CGD-H BNM 0108-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -940,33 +948,29 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 14:A. HIGH RISK HAZARD AREA25-12-00N 092-58-00W,25-31-00N 093-52-00W,25-42-00N 095-24-00W,26-02-00N 096-32-00W,26-04-00N 096-49-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-41-00N 096-47-00W,25-02-00N 095-05-00W,24-29-00N 094-08-00W,24-20-00N 093-32-00W,24-25-00N 092-52-00W AND24-45-00N 092-43-00W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-04-00N 096-49-00W,26-01-00N 096-17-00W,26-01-00N 095-12-00W,25-59-00N 094-36-00W,25-59-00N 094-05-00W,25-25-00N 093-06-00W,25-31-00N 091-46-00W,23-32-00N 088-52-00W,23-04-00N 088-33-00W,22-03-00N 086-24-00W,21-38-00N 084-59-00W,20-59-00N 082-38-00W,20-43-00N 081-42-00W,20-07-00N 079-44-00W,19-46-00N 078-47-00W,19-23-00N 078-04-00W,19-19-00N 078-18-00W,19-34-00N 079-19-00W,19-44-00N 079-44-00W,20-12-00N 081-13-00W,20-43-00N 083-13-00W,21-06-00N 084-54-00W,21-43-00N 086-42-00W,21-59-00N 087-26-00W,22-39-00N 089-10-00W,22-45-00N 089-41-00W,22-58-00N 092-36-00W,24-18-00N 095-02-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:28/1215Z SEP 26 TO 28/1414Z SEP 2629/1215Z SEP 26 TO 29/1414Z SEP 2630/1215Z SEP 26 TO 30/1414Z SEP 2601/1215Z OCT 26 TO 01/1414Z OCT 2602/1215Z OCT 26 TO 02/1414Z OCT 2603/1215Z OCT 26 TO 03/1414Z OCT 2604/1215Z OCT 26 TO 04/1414Z OCT 263. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//041514Z OCT 26// BT</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46283.699375</v>
+        <v>46290.59799768519</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -975,234 +979,198 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>587</v>
+        <v>481</v>
       </c>
       <c r="K12" t="n">
-        <v>593</v>
+        <v>484</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" s="2" t="n">
-        <v>46284</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>46285</v>
-      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Cumbyville</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46282.57303240741</v>
+        <v>46288.66804398148</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>691</v>
-      </c>
-      <c r="K13" t="n">
-        <v>701.2</v>
-      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" s="2" t="n">
-        <v>46277</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>46283</v>
-      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
-        </is>
-      </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46281.77060185185</v>
+        <v>46288.45719907407</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>652</v>
-      </c>
-      <c r="K14" t="n">
-        <v>652</v>
-      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" s="2" t="n">
-        <v>46281</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>46287</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Mariners are advised to transit the area with caution.</t>
-        </is>
-      </c>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46281.41737268519</v>
+        <v>46283.699375</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>587</v>
+      </c>
+      <c r="K15" t="n">
+        <v>593</v>
+      </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="N15" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>46285</v>
+      </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Cumbyville</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46282.57303240741</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1210,11 +1178,7 @@
           <t>dredging</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>connected to above line</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Jadwin</t>
@@ -1229,19 +1193,27 @@
         <v>691</v>
       </c>
       <c r="K16" t="n">
-        <v>701</v>
+        <v>701.2</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="N16" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>46283</v>
+      </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1252,7 +1224,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46281.77060185185</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
@@ -1263,48 +1235,50 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>303</v>
+        <v>652</v>
       </c>
       <c r="K17" t="n">
-        <v>585</v>
+        <v>652</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>46278</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>12'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Mariners are advised to transit the area with caution.</t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1315,100 +1289,86 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>585</v>
-      </c>
-      <c r="K18" t="n">
-        <v>869</v>
-      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" s="2" t="n">
-        <v>46278</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>11'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>shoaling</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>connected to above line</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>482</v>
+        <v>691</v>
       </c>
       <c r="K19" t="n">
-        <v>482</v>
+        <v>701</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
@@ -1420,7 +1380,7 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1431,51 +1391,81 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>303</v>
+      </c>
+      <c r="K20" t="n">
+        <v>585</v>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>12'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr"/>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1491,37 +1481,45 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K21" t="n">
         <v>869</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
+      <c r="N21" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>11'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46275.97677083333</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>46291</v>
-      </c>
+        <v>46277.53633101852</v>
+      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
@@ -1530,46 +1528,38 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>663</v>
+        <v>482</v>
       </c>
       <c r="K22" t="n">
-        <v>663</v>
+        <v>482</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="O22" s="2" t="n">
-        <v>46281</v>
-      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1580,14 +1570,14 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46273.435</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1610,29 +1600,21 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1663,62 +1645,88 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>n</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46268.53527777778</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
+        <v>46275.97677083333</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>46291</v>
+      </c>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>663</v>
+      </c>
+      <c r="K25" t="n">
+        <v>663</v>
+      </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46281</v>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46273.435</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1741,33 +1749,49 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>303</v>
+      </c>
+      <c r="K27" t="n">
+        <v>869</v>
+      </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
@@ -1778,21 +1802,25 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1815,21 +1843,21 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1852,21 +1880,21 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1889,21 +1917,21 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1926,21 +1954,21 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1963,21 +1991,21 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2000,21 +2028,21 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2037,21 +2065,21 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2074,21 +2102,21 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2111,21 +2139,21 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2135,50 +2163,34 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K37" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2197,34 +2209,22 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0053-26</t>
@@ -2232,63 +2232,39 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>736</v>
-      </c>
-      <c r="K39" t="n">
-        <v>736</v>
-      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2304,10 +2280,10 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>435.8</v>
+        <v>661.7</v>
       </c>
       <c r="K40" t="n">
-        <v>435.8</v>
+        <v>661.7</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
@@ -2323,7 +2299,7 @@
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2334,102 +2310,106 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
-        <v>785</v>
-      </c>
-      <c r="K41" t="n">
-        <v>785</v>
-      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O41" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>736</v>
+      </c>
+      <c r="K42" t="n">
+        <v>736</v>
+      </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="N42" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2440,14 +2420,14 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2459,14 +2439,14 @@
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>325.2</v>
+        <v>435.8</v>
       </c>
       <c r="K43" t="n">
-        <v>325.2</v>
+        <v>435.8</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
@@ -2476,13 +2456,13 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2493,60 +2473,76 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>785</v>
+      </c>
+      <c r="K44" t="n">
+        <v>785</v>
+      </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="N44" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0046-26</t>
@@ -2554,49 +2550,25 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J45" t="n">
-        <v>849</v>
-      </c>
-      <c r="K45" t="n">
-        <v>849</v>
-      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O45" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2607,14 +2579,14 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2626,14 +2598,14 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J46" t="n">
-        <v>857</v>
+        <v>325.2</v>
       </c>
       <c r="K46" t="n">
-        <v>867</v>
+        <v>325.2</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
@@ -2643,13 +2615,13 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2660,14 +2632,14 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2677,17 +2649,9 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="K47" t="n">
-        <v>10.3</v>
-      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
@@ -2696,13 +2660,13 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2713,20 +2677,18 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46234.89293981482</v>
+      </c>
+      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2745,35 +2707,35 @@
           <t>LMR</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M48" t="n">
-        <v>-90.17319999999999</v>
-      </c>
+      <c r="J48" t="n">
+        <v>849</v>
+      </c>
+      <c r="K48" t="n">
+        <v>849</v>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
       <c r="N48" s="2" t="n">
-        <v>46188</v>
+        <v>46234</v>
       </c>
       <c r="O48" s="2" t="n">
-        <v>46195</v>
+        <v>46243</v>
       </c>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2784,23 +2746,19 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
@@ -2811,10 +2769,10 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>777.7</v>
+        <v>857</v>
       </c>
       <c r="K49" t="n">
-        <v>777.7</v>
+        <v>867</v>
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
@@ -2822,42 +2780,38 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -2868,95 +2822,97 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>125.4</v>
+        <v>10.3</v>
       </c>
       <c r="K50" t="n">
-        <v>155.9</v>
+        <v>10.3</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O50" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46119.48518518519</v>
-      </c>
-      <c r="B51" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J51" t="n">
-        <v>686</v>
-      </c>
-      <c r="K51" t="n">
-        <v>686</v>
-      </c>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M51" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O51" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2967,37 +2923,37 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>348.7</v>
+        <v>777.7</v>
       </c>
       <c r="K52" t="n">
-        <v>348.7</v>
+        <v>777.7</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
@@ -3005,19 +2961,15 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
+      <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
@@ -3028,11 +2980,9 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B53" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46146.4284375</v>
+      </c>
+      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
@@ -3041,48 +2991,50 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>303</v>
+        <v>125.4</v>
       </c>
       <c r="K53" t="n">
-        <v>869</v>
+        <v>155.9</v>
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
       <c r="N53" s="2" t="n">
-        <v>46068</v>
-      </c>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
+        <v>46146</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+        </is>
+      </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3093,11 +3045,9 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B54" s="2" t="n">
-        <v>46265</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
@@ -3106,7 +3056,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3122,10 +3072,10 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>603</v>
+        <v>686</v>
       </c>
       <c r="K54" t="n">
-        <v>603</v>
+        <v>686</v>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
@@ -3135,17 +3085,17 @@
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3156,7 +3106,7 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
@@ -3167,54 +3117,46 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M55" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N55" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O55" s="2" t="n">
-        <v>46065</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="K55" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3225,12 +3167,12 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46058.58436342593</v>
-      </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" s="2" t="n">
-        <v>46068</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>N</t>
@@ -3238,7 +3180,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3254,7 +3196,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>585</v>
+        <v>303</v>
       </c>
       <c r="K56" t="n">
         <v>869</v>
@@ -3262,7 +3204,7 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
@@ -3272,14 +3214,14 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>10'6" draft, 6 barges wide</t>
+          <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3290,25 +3232,25 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46051.75101851852</v>
-      </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" s="2" t="n">
-        <v>46061</v>
-      </c>
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
@@ -3319,32 +3261,30 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="K57" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
-      <c r="N57" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -3355,12 +3295,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B58" t="inlineStr"/>
-      <c r="C58" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>N</t>
@@ -3368,48 +3306,54 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J58" t="n">
-        <v>303</v>
-      </c>
-      <c r="K58" t="n">
-        <v>585</v>
-      </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M58" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N58" s="2" t="n">
-        <v>46050</v>
-      </c>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O58" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -3420,11 +3364,11 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" s="2" t="n">
-        <v>46050</v>
+        <v>46068</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3433,7 +3377,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3449,32 +3393,32 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K59" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
       <c r="N59" s="2" t="n">
-        <v>46045</v>
+        <v>46061</v>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -3485,10 +3429,12 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" s="2" t="n">
+        <v>46061</v>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
           <t>N</t>
@@ -3496,54 +3442,48 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M60" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J60" t="n">
+        <v>303</v>
+      </c>
+      <c r="K60" t="n">
+        <v>869</v>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
       <c r="N60" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O60" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S60" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46052</v>
+      </c>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -3554,23 +3494,25 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -3581,30 +3523,32 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K61" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+      <c r="N61" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S61" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -3615,11 +3559,11 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B62" t="inlineStr"/>
       <c r="C62" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3628,7 +3572,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3647,17 +3591,17 @@
         <v>303</v>
       </c>
       <c r="K62" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
       <c r="N62" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -3669,7 +3613,7 @@
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -3680,64 +3624,259 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M63" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N63" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O63" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K64" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>303</v>
+      </c>
+      <c r="K65" t="n">
+        <v>869</v>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
         <v>46033.86975694444</v>
       </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" s="2" t="n">
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0106-26</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J63" t="n">
+      <c r="J66" t="n">
         <v>303</v>
       </c>
-      <c r="K63" t="n">
+      <c r="K66" t="n">
         <v>869</v>
       </c>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" s="2" t="n">
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr">
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="Q66" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
-      <c r="T63" t="inlineStr">
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="U66" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-10-07: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U64"/>
+  <dimension ref="A1:U68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,34 +541,26 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46301.50265046296</v>
+        <v>46302.45918981481</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0066-26</t>
+          <t>CGD-H BNM 0117-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>785</v>
-      </c>
-      <c r="K2" t="n">
-        <v>785</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -577,27 +569,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>LMR 7851. DREDGE MIDWAY REQUESTS SLOW BELL NORTHBOUND AND SOUTHBOUND IVO MM 785 LMR.2. MARINERS ARE REQUESTED NOT TO MOOR UP BY THE PIPELINE.3. DREDGE MIDWAY CAN BE CONTACTED VIA VHF CHANNEL 13 OR 71.ALL MARINERS ARE REQUESTED TO TRANSIT THE AREA WITH CAUTION BT</t>
+          <t>WITH THE APPROACH OF TROPICAL STORM ISAIAS, PROJECTED TO BECOME HURRICANE ISAIAS, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL WEATHER MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//102200Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46300.76416666667</v>
+        <v>46301.63203703704</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0114-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -616,29 +608,25 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010400Z NOV 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0058-26 DTG 111759Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46300.76378472222</v>
+        <v>46301.62190972222</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0113-26</t>
+          <t>CGD-H BNM 0116-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -659,27 +647,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>BETWEEN 07OCT2026 AND 18OCT2026, THE U.S. NAVY WILL CONDUCT DAILY UNEXPLODED ORDINANCE EXERCISES IN THE GULF OF AMERICA, NEAR APPROXIMATE POSITIONS 29-57-17.22N 086-03-03.36W AND 30-00-45.24N 085-44-27.30W. MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL CRAFT.CANCEL AT//190500Z OCT 26// BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-43-54.06N 096-58-39.60W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46300.76337962963</v>
+        <v>46301.62096064815</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0112-26</t>
+          <t>CGD-H BNM 0115-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -698,37 +686,49 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0112-26 DTG 051544Z OCT 262. USAF MISSION CANCELLED. BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-41-06.12N 97-00-12.00W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46300.54696759259</v>
+        <v>46301.50265046296</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0112-26</t>
+          <t>SEC LMR BNM 0066-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>785</v>
+      </c>
+      <c r="K6" t="n">
+        <v>785</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -737,27 +737,27 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>ON 06OCT2026, BETWEEN 1300Z AND 1700Z, THE USAF WILL CONDUCT MUNITION LAUNCHES IN THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-16-50N 086-49-22W,30-10-09N 086-47-57W,29-51-08N 086-13-40W AND29-57-48N 086-32-54W.BACK-UP DATES INCLUDE 07OCT2026, 08OCT2026, 09OCT2026 AND 13OCT2026. MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//131800Z OCT 26// BT</t>
+          <t>LMR 7851. DREDGE MIDWAY REQUESTS SLOW BELL NORTHBOUND AND SOUTHBOUND IVO MM 785 LMR.2. MARINERS ARE REQUESTED NOT TO MOOR UP BY THE PIPELINE.3. DREDGE MIDWAY CAN BE CONTACTED VIA VHF CHANNEL 13 OR 71.ALL MARINERS ARE REQUESTED TO TRANSIT THE AREA WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46296.38649305556</v>
+        <v>46300.76416666667</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>CGD-H BNM 0114-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -776,90 +776,70 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010400Z NOV 26// BT</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46293.87546296296</v>
+        <v>46300.76378472222</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>CGD-H BNM 0113-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>408</v>
-      </c>
-      <c r="K8" t="n">
-        <v>486.2</v>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" s="2" t="n">
-        <v>46293</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>46295</v>
-      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>BETWEEN 07OCT2026 AND 18OCT2026, THE U.S. NAVY WILL CONDUCT DAILY UNEXPLODED ORDINANCE EXERCISES IN THE GULF OF AMERICA, NEAR APPROXIMATE POSITIONS 29-57-17.22N 086-03-03.36W AND 30-00-45.24N 085-44-27.30W. MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL CRAFT.CANCEL AT//190500Z OCT 26// BT</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46293.48231481481</v>
+        <v>46300.76337962963</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>CGD-H BNM 0112-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -882,90 +862,62 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0112-26 DTG 051544Z OCT 262. USAF MISSION CANCELLED. BT</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46290.59799768519</v>
+        <v>46300.54696759259</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>CGD-H BNM 0112-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>481</v>
-      </c>
-      <c r="K10" t="n">
-        <v>484</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" s="2" t="n">
-        <v>46290</v>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>46291</v>
-      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Lake Providence</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 06OCT2026, BETWEEN 1300Z AND 1700Z, THE USAF WILL CONDUCT MUNITION LAUNCHES IN THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-16-50N 086-49-22W,30-10-09N 086-47-57W,29-51-08N 086-13-40W AND29-57-48N 086-32-54W.BACK-UP DATES INCLUDE 07OCT2026, 08OCT2026, 09OCT2026 AND 13OCT2026. MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//131800Z OCT 26// BT</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46288.66804398148</v>
+        <v>46296.38649305556</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -988,7 +940,7 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
+          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -999,113 +951,109 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46288.45719907407</v>
+        <v>46293.87546296296</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>408</v>
+      </c>
+      <c r="K12" t="n">
+        <v>486.2</v>
+      </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="N12" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>46295</v>
+      </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
+          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46283.699375</v>
+        <v>46293.48231481481</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>587</v>
-      </c>
-      <c r="K13" t="n">
-        <v>593</v>
-      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" s="2" t="n">
-        <v>46284</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>46285</v>
-      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Cumbyville</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46282.57303240741</v>
+        <v>46290.59799768519</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
@@ -1116,7 +1064,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1136,30 +1084,30 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>691</v>
+        <v>481</v>
       </c>
       <c r="K14" t="n">
-        <v>701.2</v>
+        <v>484</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>46277</v>
+        <v>46290</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>46283</v>
+        <v>46291</v>
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Commerce</t>
+          <t>Lake Providence</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1170,15 +1118,11 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46281.77060185185</v>
+        <v>46288.66804398148</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0060-26</t>
@@ -1186,63 +1130,43 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>652</v>
-      </c>
-      <c r="K15" t="n">
-        <v>652</v>
-      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" s="2" t="n">
-        <v>46281</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>46287</v>
-      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Mariners are advised to transit the area with caution.</t>
-        </is>
-      </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46281.41737268519</v>
+        <v>46288.45719907407</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1265,7 +1189,7 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1276,18 +1200,18 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46283.699375</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1295,11 +1219,7 @@
           <t>dredging</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>connected to above line</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Jadwin</t>
@@ -1311,22 +1231,30 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>691</v>
+        <v>587</v>
       </c>
       <c r="K17" t="n">
-        <v>701</v>
+        <v>593</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="N17" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>46285</v>
+      </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Cumbyville</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1337,7 +1265,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46282.57303240741</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -1348,48 +1276,50 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>585</v>
+        <v>691</v>
       </c>
       <c r="K18" t="n">
-        <v>869</v>
+        <v>701.2</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>46278</v>
-      </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>11'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr"/>
+        <v>46277</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Commerce</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1400,7 +1330,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46281.77060185185</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -1411,48 +1341,50 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>303</v>
+        <v>652</v>
       </c>
       <c r="K19" t="n">
-        <v>585</v>
+        <v>652</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>46278</v>
-      </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>12'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Mariners are advised to transit the area with caution.</t>
+        </is>
+      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1463,38 +1395,26 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>482</v>
-      </c>
-      <c r="K20" t="n">
-        <v>482</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
@@ -1505,37 +1425,57 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46280.38037037037</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>connected to above line</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>691</v>
+      </c>
+      <c r="K21" t="n">
+        <v>701</v>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
@@ -1546,21 +1486,29 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr"/>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1576,37 +1524,45 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K22" t="n">
         <v>869</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>11'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46275.97677083333</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>46291</v>
-      </c>
+        <v>46278.72424768518</v>
+      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
@@ -1615,46 +1571,48 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>663</v>
+        <v>303</v>
       </c>
       <c r="K23" t="n">
-        <v>663</v>
+        <v>585</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>46281</v>
-      </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
+        <v>46278</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>12'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1665,26 +1623,38 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46273.435</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>482</v>
+      </c>
+      <c r="K24" t="n">
+        <v>482</v>
+      </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
@@ -1695,7 +1665,7 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1706,15 +1676,11 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0055-26</t>
@@ -1722,22 +1688,14 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>303</v>
-      </c>
-      <c r="K25" t="n">
-        <v>869</v>
-      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
@@ -1748,37 +1706,41 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>303</v>
+      </c>
+      <c r="K26" t="n">
+        <v>869</v>
+      </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
@@ -1789,58 +1751,88 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr"/>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46265.53005787037</v>
-      </c>
-      <c r="B27" t="inlineStr"/>
+        <v>46275.97677083333</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>46291</v>
+      </c>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>663</v>
+      </c>
+      <c r="K27" t="n">
+        <v>663</v>
+      </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="N27" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>46281</v>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr"/>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46273.435</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1863,33 +1855,49 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr"/>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>303</v>
+      </c>
+      <c r="K29" t="n">
+        <v>869</v>
+      </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
@@ -1900,21 +1908,25 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr"/>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1937,21 +1949,21 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1974,21 +1986,21 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2011,21 +2023,21 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2048,14 +2060,14 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
@@ -2092,14 +2104,14 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2122,21 +2134,21 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2159,21 +2171,21 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2196,21 +2208,21 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2220,50 +2232,34 @@
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K38" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2282,98 +2278,62 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J40" t="n">
-        <v>736</v>
-      </c>
-      <c r="K40" t="n">
-        <v>736</v>
-      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2383,120 +2343,92 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K41" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>785</v>
+        <v>661.7</v>
       </c>
       <c r="K42" t="n">
-        <v>785</v>
+        <v>661.7</v>
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O42" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2510,82 +2442,98 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>AL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J44" t="n">
-        <v>325.2</v>
+        <v>736</v>
       </c>
       <c r="K44" t="n">
-        <v>325.2</v>
+        <v>736</v>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="N44" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2595,9 +2543,17 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K45" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
@@ -2606,13 +2562,13 @@
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2623,7 +2579,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
@@ -2634,7 +2590,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2654,34 +2610,30 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>849</v>
+        <v>785</v>
       </c>
       <c r="K46" t="n">
-        <v>849</v>
+        <v>785</v>
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" s="2" t="n">
-        <v>46234</v>
+        <v>46244</v>
       </c>
       <c r="O46" s="2" t="n">
-        <v>46243</v>
+        <v>46251</v>
       </c>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2692,67 +2644,55 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>857</v>
-      </c>
-      <c r="K47" t="n">
-        <v>867</v>
-      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2768,10 +2708,10 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>10.3</v>
+        <v>325.2</v>
       </c>
       <c r="K48" t="n">
-        <v>10.3</v>
+        <v>325.2</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
@@ -2787,7 +2727,7 @@
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2798,78 +2738,52 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B49" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46238.74310185185</v>
+      </c>
+      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M49" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N49" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O49" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
@@ -2880,42 +2794,54 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>777.7</v>
+        <v>849</v>
       </c>
       <c r="K50" t="n">
-        <v>777.7</v>
+        <v>849</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="N50" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2926,102 +2852,86 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>125.4</v>
+        <v>857</v>
       </c>
       <c r="K51" t="n">
-        <v>155.9</v>
+        <v>867</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
-      <c r="N51" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O51" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>686</v>
+        <v>10.3</v>
       </c>
       <c r="K52" t="n">
-        <v>686</v>
+        <v>10.3</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
@@ -3031,30 +2941,28 @@
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46093.45828703704</v>
-      </c>
-      <c r="B53" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
@@ -3063,46 +2971,54 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J53" t="n">
-        <v>348.7</v>
-      </c>
-      <c r="K53" t="n">
-        <v>348.7</v>
-      </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M53" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3113,25 +3029,23 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B54" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46160.52664351852</v>
+      </c>
+      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
@@ -3142,32 +3056,26 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>303</v>
+        <v>777.7</v>
       </c>
       <c r="K54" t="n">
-        <v>869</v>
+        <v>777.7</v>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
@@ -3178,59 +3086,61 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B55" s="2" t="n">
-        <v>46265</v>
-      </c>
+        <v>46146.4284375</v>
+      </c>
+      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>603</v>
+        <v>125.4</v>
       </c>
       <c r="K55" t="n">
-        <v>603</v>
+        <v>155.9</v>
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
+      <c r="N55" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P55" t="inlineStr"/>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
@@ -3241,65 +3151,57 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M56" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N56" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O56" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J56" t="n">
+        <v>686</v>
+      </c>
+      <c r="K56" t="n">
+        <v>686</v>
+      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3310,12 +3212,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B57" t="inlineStr"/>
-      <c r="C57" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>N</t>
@@ -3323,48 +3223,46 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>585</v>
+        <v>348.7</v>
       </c>
       <c r="K57" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
-      <c r="N57" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -3375,12 +3273,12 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46051.75101851852</v>
-      </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" s="2" t="n">
-        <v>46061</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>N</t>
@@ -3388,7 +3286,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3412,7 +3310,7 @@
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
       <c r="N58" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
@@ -3429,7 +3327,7 @@
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -3440,25 +3338,25 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46050.44465277778</v>
-      </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" s="2" t="n">
-        <v>46052</v>
-      </c>
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
@@ -3469,32 +3367,30 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="K59" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
-      <c r="N59" s="2" t="n">
-        <v>46050</v>
-      </c>
+      <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -3505,12 +3401,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B60" t="inlineStr"/>
-      <c r="C60" s="2" t="n">
-        <v>46050</v>
-      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>N</t>
@@ -3518,48 +3412,54 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J60" t="n">
-        <v>303</v>
-      </c>
-      <c r="K60" t="n">
-        <v>585</v>
-      </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M60" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N60" s="2" t="n">
-        <v>46045</v>
-      </c>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q60" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -3570,10 +3470,12 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>N</t>
@@ -3581,54 +3483,48 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M61" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J61" t="n">
+        <v>585</v>
+      </c>
+      <c r="K61" t="n">
+        <v>869</v>
+      </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
       <c r="N61" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O61" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S61" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46061</v>
+      </c>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>10'6" draft, 6 barges wide</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -3639,23 +3535,25 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" s="2" t="n">
+        <v>46061</v>
+      </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
@@ -3666,30 +3564,32 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K62" t="n">
-        <v>538.7</v>
+        <v>869</v>
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -3700,11 +3600,11 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3713,7 +3613,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3732,17 +3632,17 @@
         <v>303</v>
       </c>
       <c r="K63" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
       <c r="N63" s="2" t="n">
-        <v>46037</v>
+        <v>46050</v>
       </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -3754,7 +3654,7 @@
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -3765,11 +3665,11 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" s="2" t="n">
-        <v>46037</v>
+        <v>46050</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3778,7 +3678,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3797,17 +3697,17 @@
         <v>303</v>
       </c>
       <c r="K64" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
       <c r="N64" s="2" t="n">
-        <v>46034</v>
+        <v>46045</v>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -3819,10 +3719,270 @@
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr">
         <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M65" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N65" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O65" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K66" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>303</v>
+      </c>
+      <c r="K67" t="n">
+        <v>869</v>
+      </c>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>303</v>
+      </c>
+      <c r="K68" t="n">
+        <v>869</v>
+      </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="U68" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-10-08: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U68"/>
+  <dimension ref="A1:U74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,19 +541,19 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46302.45918981481</v>
+        <v>46303.485625</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0117-26</t>
+          <t>SEC LMR BNM 0063-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -567,29 +567,25 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF TROPICAL STORM ISAIAS, PROJECTED TO BECOME HURRICANE ISAIAS, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL WEATHER MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//102200Z OCT 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0063-26 DTG 011747Z OCT 26 BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46301.63203703704</v>
+        <v>46303.48527777778</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0063-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -612,21 +608,21 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0058-26 DTG 111759Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0063-26 DTG 011747Z OCT 26 BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46301.62190972222</v>
+        <v>46303.48493055555</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0116-26</t>
+          <t>SEC LMR BNM 0064-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -645,29 +641,25 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-43-54.06N 096-58-39.60W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0064-26 DTG 011740Z OCT 26 BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46301.62096064815</v>
+        <v>46303.48447916667</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0115-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -686,78 +678,62 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-41-06.12N 97-00-12.00W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0059-26 DTG 121519Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46301.50265046296</v>
+        <v>46303.47424768518</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0066-26</t>
+          <t>CGD-H BNM 0116-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>785</v>
-      </c>
-      <c r="K6" t="n">
-        <v>785</v>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>LMR 7851. DREDGE MIDWAY REQUESTS SLOW BELL NORTHBOUND AND SOUTHBOUND IVO MM 785 LMR.2. MARINERS ARE REQUESTED NOT TO MOOR UP BY THE PIPELINE.3. DREDGE MIDWAY CAN BE CONTACTED VIA VHF CHANNEL 13 OR 71.ALL MARINERS ARE REQUESTED TO TRANSIT THE AREA WITH CAUTION BT</t>
+          <t>1. CANCEL CGD-H BNM 0116-26 DTG 061427Z OCT 262. BUOY RECOVERED BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46300.76416666667</v>
+        <v>46303.47325231481</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0114-26</t>
+          <t>CGD-H BNM 0115-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -776,34 +752,30 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010400Z NOV 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0115-26 DTG 061424Z OCT 262. BUOY RECOVERED BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46300.76378472222</v>
+        <v>46302.45918981481</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0113-26</t>
+          <t>CGD-H BNM 0117-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -819,27 +791,27 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>BETWEEN 07OCT2026 AND 18OCT2026, THE U.S. NAVY WILL CONDUCT DAILY UNEXPLODED ORDINANCE EXERCISES IN THE GULF OF AMERICA, NEAR APPROXIMATE POSITIONS 29-57-17.22N 086-03-03.36W AND 30-00-45.24N 085-44-27.30W. MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL CRAFT.CANCEL AT//190500Z OCT 26// BT</t>
+          <t>WITH THE APPROACH OF TROPICAL STORM ISAIAS, PROJECTED TO BECOME HURRICANE ISAIAS, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL WEATHER MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//102200Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46300.76337962963</v>
+        <v>46301.63203703704</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0112-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -862,21 +834,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0112-26 DTG 051544Z OCT 262. USAF MISSION CANCELLED. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0058-26 DTG 111759Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46300.54696759259</v>
+        <v>46301.62190972222</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0112-26</t>
+          <t>CGD-H BNM 0116-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -897,27 +869,27 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>ON 06OCT2026, BETWEEN 1300Z AND 1700Z, THE USAF WILL CONDUCT MUNITION LAUNCHES IN THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-16-50N 086-49-22W,30-10-09N 086-47-57W,29-51-08N 086-13-40W AND29-57-48N 086-32-54W.BACK-UP DATES INCLUDE 07OCT2026, 08OCT2026, 09OCT2026 AND 13OCT2026. MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//131800Z OCT 26// BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-43-54.06N 096-58-39.60W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46296.38649305556</v>
+        <v>46301.62096064815</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>CGD-H BNM 0115-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -936,33 +908,29 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-41-06.12N 97-00-12.00W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46293.87546296296</v>
+        <v>46301.50265046296</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>SEC LMR BNM 0066-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -971,55 +939,47 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>408</v>
+        <v>785</v>
       </c>
       <c r="K12" t="n">
-        <v>486.2</v>
+        <v>785</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" s="2" t="n">
-        <v>46293</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>46295</v>
-      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>LMR 7851. DREDGE MIDWAY REQUESTS SLOW BELL NORTHBOUND AND SOUTHBOUND IVO MM 785 LMR.2. MARINERS ARE REQUESTED NOT TO MOOR UP BY THE PIPELINE.3. DREDGE MIDWAY CAN BE CONTACTED VIA VHF CHANNEL 13 OR 71.ALL MARINERS ARE REQUESTED TO TRANSIT THE AREA WITH CAUTION BT</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46293.48231481481</v>
+        <v>46300.76416666667</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>CGD-H BNM 0114-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1038,94 +998,70 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010400Z NOV 26// BT</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46290.59799768519</v>
+        <v>46300.76378472222</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0061-26</t>
+          <t>CGD-H BNM 0113-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>481</v>
-      </c>
-      <c r="K14" t="n">
-        <v>484</v>
-      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" s="2" t="n">
-        <v>46290</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>46291</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Lake Providence</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>BETWEEN 07OCT2026 AND 18OCT2026, THE U.S. NAVY WILL CONDUCT DAILY UNEXPLODED ORDINANCE EXERCISES IN THE GULF OF AMERICA, NEAR APPROXIMATE POSITIONS 29-57-17.22N 086-03-03.36W AND 30-00-45.24N 085-44-27.30W. MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL CRAFT.CANCEL AT//190500Z OCT 26// BT</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46288.66804398148</v>
+        <v>46300.76337962963</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>CGD-H BNM 0112-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1148,25 +1084,21 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0112-26 DTG 051544Z OCT 262. USAF MISSION CANCELLED. BT</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46288.45719907407</v>
+        <v>46300.54696759259</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>CGD-H BNM 0112-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1185,87 +1117,63 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 06OCT2026, BETWEEN 1300Z AND 1700Z, THE USAF WILL CONDUCT MUNITION LAUNCHES IN THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-16-50N 086-49-22W,30-10-09N 086-47-57W,29-51-08N 086-13-40W AND29-57-48N 086-32-54W.BACK-UP DATES INCLUDE 07OCT2026, 08OCT2026, 09OCT2026 AND 13OCT2026. MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//131800Z OCT 26// BT</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46283.699375</v>
+        <v>46296.38649305556</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>587</v>
-      </c>
-      <c r="K17" t="n">
-        <v>593</v>
-      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" s="2" t="n">
-        <v>46284</v>
-      </c>
-      <c r="O17" s="2" t="n">
-        <v>46285</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Cumbyville</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46282.57303240741</v>
+        <v>46293.87546296296</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -1276,7 +1184,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0062-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1296,30 +1204,26 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>691</v>
+        <v>408</v>
       </c>
       <c r="K18" t="n">
-        <v>701.2</v>
+        <v>486.2</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>46277</v>
+        <v>46293</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>46283</v>
+        <v>46295</v>
       </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Commerce</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
+          <t>LMR MM 408-4861.DREDGE JADWIN WILL BEGIN DREDGING OPERATIONS BETWEEN LMR MM 408-486.2.VESSEL TRAFFIC WILL BE RESTRICTED TO ONE WAY TRAFFIC UNTIL SEPTEMBER 30. DREDGE JADWIN WILL BE MAINTAINING THE QUEUE.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157BT BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1330,152 +1234,132 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46281.77060185185</v>
+        <v>46293.48231481481</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0060-26</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>652</v>
-      </c>
-      <c r="K19" t="n">
-        <v>652</v>
-      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" s="2" t="n">
-        <v>46281</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>46287</v>
-      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Mariners are advised to transit the area with caution.</t>
-        </is>
-      </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0061-26 DTG 251710Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46281.41737268519</v>
+        <v>46290.59799768519</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0061-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>481</v>
+      </c>
+      <c r="K20" t="n">
+        <v>484</v>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="N20" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>46291</v>
+      </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Lake Providence</t>
+        </is>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO LAKE PROVIDENCE, BETWEEN LMR MM 481-4842.VESSEL TRAFFIC WILL BE STOPPED FROM 1030 SEPTEMBER 25TH THROUGH 1030 SEPTEMBER 26TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46280.38037037037</v>
+        <v>46288.66804398148</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0056-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>connected to above line</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Jadwin</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>691</v>
-      </c>
-      <c r="K21" t="n">
-        <v>701</v>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
@@ -1486,81 +1370,59 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0060-26 DTG 162218Z SEP 26</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46288.45719907407</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>585</v>
-      </c>
-      <c r="K22" t="n">
-        <v>869</v>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" s="2" t="n">
-        <v>46278</v>
-      </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>11'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0056-26 DTG 151249Z SEP 26</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46278.72424768518</v>
+        <v>46283.699375</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
@@ -1571,48 +1433,50 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-2</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>303</v>
+        <v>587</v>
       </c>
       <c r="K23" t="n">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>46278</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>12'6" draft. 7 barges wide.</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
+        <v>46284</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Cumbyville</t>
+        </is>
+      </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
+          <t>1.DREDGE JADWIN WILL BEGIN WORK IVO CUMBYVILLE AT 6 AM ON SEPTEMBER 19TH.2.TO FACILITATE SAFE WORK, VESSEL TRAFFIC WILL BE STOPPED AT MM 587-593 LMR, FROM 6AM ON SEPTEMBER 19TH THROUGH 6PM ON SEPTEMBER 20TH.3.DREDGE JADWIN WILL CLEAR THE QUEUE AFTER COMPLETION. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.4.TO ENTER THE QUEUE, CONTACT DREDGE JADWIN VIA VHF-FM CH 13 OR BY TELEPHONE AT 601-618-2157. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1623,7 +1487,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46277.53633101852</v>
+        <v>46282.57303240741</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
@@ -1634,38 +1498,50 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0056-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Jadwin</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>482</v>
+        <v>691</v>
       </c>
       <c r="K24" t="n">
-        <v>482</v>
+        <v>701.2</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="N24" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>46283</v>
+      </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Commerce</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.DREDGE JADWIN IS WORKING IVO COMMERCE, BETWEEN LMR MM 691-701.2.VESSEL TRAFFIC WILL BE STOPPED FROM NOON SEPTEMBER 17TH THROUGH NOON SEPTEMBER 18TH TO FACILITATE SAFE WORK. DREDGE JADWIN WILL CLEAR THE QUEUE AFTER WORK IS COMPLETED.3.ALL MARINERS DESIRING TO TRANSIT THE AREA MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4.UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1676,71 +1552,91 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46277.09849537037</v>
+        <v>46281.77060185185</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0060-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>652</v>
+      </c>
+      <c r="K25" t="n">
+        <v>652</v>
+      </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46287</v>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Mariners are advised to transit the area with caution.</t>
+        </is>
+      </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr"/>
+          <t>1. Dredge MIDWAY will be conducting dredging operations IVO MM 652 LMR until September 22nd, 24 hours a day, 7 days a week.2. Mariners can contact the M/V MIDWAY on channel 71 and 13, or phone number 314-550-0520.3. Mariners are advised to transit the area with caution. BT</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46276.67863425926</v>
+        <v>46281.41737268519</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J26" t="n">
-        <v>303</v>
-      </c>
-      <c r="K26" t="n">
-        <v>869</v>
-      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
@@ -1751,31 +1647,29 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0057-26 DTG 110131Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46275.97677083333</v>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>46291</v>
-      </c>
+        <v>46280.38037037037</v>
+      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0057-26</t>
+          <t>SEC LMR BNM 0056-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1783,10 +1677,14 @@
           <t>dredging</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>connected to above line</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Midway</t>
+          <t>Jadwin</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1795,26 +1693,22 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>663</v>
+        <v>691</v>
       </c>
       <c r="K27" t="n">
-        <v>663</v>
+        <v>701</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" s="2" t="n">
-        <v>46275</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>46281</v>
-      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. COMMENCING SEPTEMBER 12TH, 2026 AT 0600, THE DREDGE JADWIN WILL BE WORKING IVO COMMERCE, BETWEEN LMR MM 691-701. ALL VESSEL TRAFFIC WILL BE STOPPED FOR AN INITIAL CLOSURE PERIOD OF APPROXIMATELY 36 HOURS, FOLLOWED BY ROLLING CLOSURES AS NEEDED.2. DREDGE JADWIN WILL PASS TRAFFIC DURING OPERATIONS IF SAFE PASSAGE CAN BE MADE; IF NOT, DREDGE JADWIN WILL CLEAR THE QUEUE UPON COMPLETION OF THE 36-HOUR PERIOD.3. ALL MARINERS DESIRING TO TRANSIT MUST CONTACT DREDGE JADWIN TO ENTER THE QUEUE VIA VHF-FM CH 13 OR 16, OR BY TELEPHONE AT 601-618-2157.4. UPON APPROVAL TO TRANSIT, MARINERS ARE REQUESTED TO TRANSIT THE AREA AT SAFE SPEED AND PROCEED WITH CAUTION.BTCANCEL AT//291250Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1825,37 +1719,59 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46273.435</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>585</v>
+      </c>
+      <c r="K28" t="n">
+        <v>869</v>
+      </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+      <c r="N28" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>11'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1866,18 +1782,18 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46268.97141203703</v>
+        <v>46278.72424768518</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0055-26</t>
+          <t>SEC LMR BNM 0058-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1896,49 +1812,71 @@
         <v>303</v>
       </c>
       <c r="K29" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
+      <c r="N29" s="2" t="n">
+        <v>46278</v>
+      </c>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>10'6" draft. 4 barges wide and 6 long on loads. 6 barges wide and 7 long overall.</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>12'6" draft. 7 barges wide.</t>
+        </is>
+      </c>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+          <t>LMR MM 303-869Mariners be advised that MSIB 26-10 low-water restrictions will remain in effect for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:â€¢ Barge drafts not to exceed 12'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 4 wide and 6 long max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall.BT BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46268.53527777778</v>
+        <v>46277.53633101852</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>482</v>
+      </c>
+      <c r="K30" t="n">
+        <v>482</v>
+      </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
@@ -1949,21 +1887,25 @@
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr"/>
+          <t>1. THE CG RCVD A REPORT OF SHOALING IVO MM 482 LMR.2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46277.09849537037</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1986,33 +1928,41 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. CANCEL SEC LMR BNM 0055-26 DTG 032121Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46276.67863425926</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>303</v>
+      </c>
+      <c r="K32" t="n">
+        <v>869</v>
+      </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
@@ -2023,58 +1973,88 @@
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr"/>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-11 which updates low-water restrictions on September 14th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Barge drafts not to exceed 11'.â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-480:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 480-303:â€¢ Barge drafts not to exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide and 6 long for max on loads.â€¢ Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46265.52792824074</v>
-      </c>
-      <c r="B33" t="inlineStr"/>
+        <v>46275.97677083333</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>46291</v>
+      </c>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR BNM 0057-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>663</v>
+      </c>
+      <c r="K33" t="n">
+        <v>663</v>
+      </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
+      <c r="N33" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>46281</v>
+      </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr"/>
+          <t>LMR MM 6631. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS IVO MM 663 LMR UNTIL SEPTEMBER 15. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46273.435</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2097,33 +2077,49 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr"/>
+          <t>1. CANCEL CGD-H BNM 0095-26 DTG 021625Z SEP 26 BT</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>303</v>
+      </c>
+      <c r="K35" t="n">
+        <v>869</v>
+      </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
@@ -2134,21 +2130,25 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr"/>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2171,21 +2171,21 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2208,21 +2208,21 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2245,21 +2245,21 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2282,21 +2282,21 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2319,21 +2319,21 @@
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2356,21 +2356,21 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2380,50 +2380,34 @@
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K42" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U42" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2442,98 +2426,62 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J44" t="n">
-        <v>736</v>
-      </c>
-      <c r="K44" t="n">
-        <v>736</v>
-      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O44" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2543,120 +2491,76 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J45" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K45" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U45" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J46" t="n">
-        <v>785</v>
-      </c>
-      <c r="K46" t="n">
-        <v>785</v>
-      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O46" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>Osceola Harbor</t>
-        </is>
-      </c>
+      <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2674,25 +2578,21 @@
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
-        </is>
-      </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2704,14 +2604,14 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J48" t="n">
-        <v>325.2</v>
+        <v>661.7</v>
       </c>
       <c r="K48" t="n">
-        <v>325.2</v>
+        <v>661.7</v>
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
@@ -2721,13 +2621,13 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -2738,14 +2638,14 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2766,13 +2666,13 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
@@ -2783,7 +2683,7 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr"/>
@@ -2794,7 +2694,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2814,34 +2714,30 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>849</v>
+        <v>736</v>
       </c>
       <c r="K50" t="n">
-        <v>849</v>
+        <v>736</v>
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" s="2" t="n">
-        <v>46234</v>
+        <v>46251</v>
       </c>
       <c r="O50" s="2" t="n">
-        <v>46243</v>
+        <v>46257</v>
       </c>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
@@ -2852,14 +2748,14 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2875,10 +2771,10 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>857</v>
+        <v>435.8</v>
       </c>
       <c r="K51" t="n">
-        <v>867</v>
+        <v>435.8</v>
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
@@ -2894,7 +2790,7 @@
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
@@ -2905,120 +2801,102 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>10.3</v>
+        <v>785</v>
       </c>
       <c r="K52" t="n">
-        <v>10.3</v>
+        <v>785</v>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="N52" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B53" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46244.30862268519</v>
+      </c>
+      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M53" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N53" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O53" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
@@ -3029,37 +2907,33 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>777.7</v>
+        <v>325.2</v>
       </c>
       <c r="K54" t="n">
-        <v>777.7</v>
+        <v>325.2</v>
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
@@ -3067,91 +2941,71 @@
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J55" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K55" t="n">
-        <v>155.9</v>
-      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O55" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
@@ -3162,46 +3016,54 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J56" t="n">
-        <v>686</v>
+        <v>849</v>
       </c>
       <c r="K56" t="n">
-        <v>686</v>
+        <v>849</v>
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
+      <c r="N56" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
@@ -3212,37 +3074,33 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>348.7</v>
+        <v>857</v>
       </c>
       <c r="K57" t="n">
-        <v>348.7</v>
+        <v>867</v>
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
@@ -3252,145 +3110,137 @@
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>"Possible shoaling," transit area with caution</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B58" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J58" t="n">
-        <v>303</v>
+        <v>10.3</v>
       </c>
       <c r="K58" t="n">
-        <v>869</v>
+        <v>10.3</v>
       </c>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
-      <c r="N58" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46186.8905787037</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>46265</v>
+        <v>46199</v>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J59" t="n">
-        <v>603</v>
-      </c>
-      <c r="K59" t="n">
-        <v>603</v>
-      </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M59" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O59" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -3401,65 +3251,53 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M60" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N60" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O60" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J60" t="n">
+        <v>777.7</v>
+      </c>
+      <c r="K60" t="n">
+        <v>777.7</v>
+      </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
+      <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U60" t="inlineStr">
@@ -3470,12 +3308,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>N</t>
@@ -3483,48 +3319,50 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>585</v>
+        <v>125.4</v>
       </c>
       <c r="K61" t="n">
-        <v>869</v>
+        <v>155.9</v>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
       <c r="N61" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q61" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
+        <v>46146</v>
+      </c>
+      <c r="O61" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+        </is>
+      </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U61" t="inlineStr">
@@ -3535,25 +3373,23 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B62" t="inlineStr"/>
-      <c r="C62" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
@@ -3564,32 +3400,30 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K62" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
-      <c r="N62" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T62" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U62" t="inlineStr">
@@ -3600,12 +3434,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B63" t="inlineStr"/>
-      <c r="C63" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>N</t>
@@ -3613,48 +3445,46 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J63" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K63" t="n">
-        <v>585</v>
+        <v>348.7</v>
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
-      <c r="N63" s="2" t="n">
-        <v>46050</v>
-      </c>
+      <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T63" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U63" t="inlineStr">
@@ -3665,12 +3495,12 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46045.53974537037</v>
-      </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" s="2" t="n">
-        <v>46050</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>N</t>
@@ -3678,7 +3508,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3697,17 +3527,17 @@
         <v>303</v>
       </c>
       <c r="K64" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
       <c r="N64" s="2" t="n">
-        <v>46045</v>
+        <v>46068</v>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -3719,7 +3549,7 @@
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
@@ -3730,65 +3560,59 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="B65" t="inlineStr"/>
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>46265</v>
+      </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M65" t="n">
-        <v>-90.10785143484679</v>
-      </c>
-      <c r="N65" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O65" s="2" t="n">
-        <v>46044</v>
-      </c>
+      <c r="J65" t="n">
+        <v>603</v>
+      </c>
+      <c r="K65" t="n">
+        <v>603</v>
+      </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr">
         <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U65" t="inlineStr">
@@ -3799,57 +3623,65 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J66" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K66" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M66" t="n">
+        <v>-90.10947400000001</v>
+      </c>
+      <c r="N66" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="O66" s="2" t="n">
+        <v>46065</v>
+      </c>
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>Amrize Dock on Mckellar Lake</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
@@ -3860,11 +3692,11 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" s="2" t="n">
-        <v>46045</v>
+        <v>46068</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3873,7 +3705,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3889,7 +3721,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K67" t="n">
         <v>869</v>
@@ -3897,7 +3729,7 @@
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
       <c r="N67" s="2" t="n">
-        <v>46037</v>
+        <v>46061</v>
       </c>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
@@ -3907,14 +3739,14 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R67" t="inlineStr"/>
       <c r="S67" t="inlineStr"/>
       <c r="T67" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U67" t="inlineStr">
@@ -3925,11 +3757,11 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" s="2" t="n">
-        <v>46037</v>
+        <v>46061</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3938,7 +3770,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3962,12 +3794,12 @@
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
       <c r="N68" s="2" t="n">
-        <v>46034</v>
+        <v>46052</v>
       </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -3979,10 +3811,400 @@
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46050.44465277778</v>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0007-26</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>303</v>
+      </c>
+      <c r="K69" t="n">
+        <v>585</v>
+      </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>303</v>
+      </c>
+      <c r="K70" t="n">
+        <v>585</v>
+      </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M71" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N71" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O71" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K72" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>303</v>
+      </c>
+      <c r="K73" t="n">
+        <v>869</v>
+      </c>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>303</v>
+      </c>
+      <c r="K74" t="n">
+        <v>869</v>
+      </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="U74" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-10-09: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -1746,10 +1746,10 @@
         </is>
       </c>
       <c r="J28" t="n">
+        <v>303</v>
+      </c>
+      <c r="K28" t="n">
         <v>585</v>
-      </c>
-      <c r="K28" t="n">
-        <v>869</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>11'6" draft. 7 barges wide.</t>
+          <t>12'6" draft. 7 barges wide.</t>
         </is>
       </c>
       <c r="R28" t="inlineStr"/>
@@ -1809,10 +1809,10 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K29" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>12'6" draft. 7 barges wide.</t>
+          <t>11'6" draft. 7 barges wide.</t>
         </is>
       </c>
       <c r="R29" t="inlineStr"/>

</xml_diff>

<commit_message>
Daily pipeline 2026-10-13: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U74"/>
+  <dimension ref="A1:U77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46303.485625</v>
+        <v>46308.55574074074</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0063-26</t>
+          <t>SEC LMR BNM 0068-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -567,25 +567,29 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0063-26 DTG 011747Z OCT 26 BT</t>
+          <t>1. CONSTRUCTION WORK FOR THE I-55 BRIDGE IVO MEMPHIS, TN WILL BEGIN ON OCTOBER 19TH.2. FROM OCTOBER 19TH THROUGH NOVEMBER 2ND, THE ARKANSAS SPAN OF THE I-55 BRIDGE WILL BE CLOSED. THE ALTERNATE SPAN WILL BE PARTIALLY REDUCED IN WIDTH; MARINERS SHOULD SAIL THE EAST SIDE OF THE SPAN. THE MAIN SPAN WILL BE UNAFFECTED.3. MARINERS CAN CONTACT M/V VIRGINIA BURNS ON CH. 13 AND CH. 68 FOR MORE INFORMATION. M/V VIRGINIA BURNS WILL BE ON-SCENE DURING WORK.4.CANCEL AT TIME//030800L NOV 26//.CANCEL AT//031300Z NOV 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46303.48527777778</v>
+        <v>46308.54804398148</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0063-26</t>
+          <t>SEC LMR BNM 0067-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -595,34 +599,46 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>710</v>
+      </c>
+      <c r="K3" t="n">
+        <v>712.5</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0063-26 DTG 011747Z OCT 26 BT</t>
+          <t>1. BORING OPERATIONS ARE BEING CONDUCTED BETWEEN MM 710-712.5 LMR FROM OCTOBER 12TH THROUGH 21ST.2.DURING THIS TIME, MARINERS SHOULD EXERCISE CAUTION DURING TRANSIT AND ENSURE ONE-WAY TRAFFIC ONLY. NO MEETING, PASSING, OR OVERTAKING.3.CANCELL AT TIME//220800L OCT 26//. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46303.48493055555</v>
+        <v>46308.37226851852</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0064-26</t>
+          <t>CGD-H BNM 0118-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -641,25 +657,29 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>FL, AL, MS, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0064-26 DTG 011740Z OCT 26 BT</t>
+          <t>DUE TO THE PASSAGE OF HURRICANE ISAIAS, AIDS TO NAVIGATION AND STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGES. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46303.48447916667</v>
+        <v>46303.485625</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0059-26</t>
+          <t>SEC LMR BNM 0063-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -682,21 +702,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0059-26 DTG 121519Z SEP 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0063-26 DTG 011747Z OCT 26 BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46303.47424768518</v>
+        <v>46303.48527777778</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0116-26</t>
+          <t>SEC LMR BNM 0063-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -719,21 +739,21 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0116-26 DTG 061427Z OCT 262. BUOY RECOVERED BT</t>
+          <t>1. CANCEL SEC LMR BNM 0063-26 DTG 011747Z OCT 26 BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46303.47325231481</v>
+        <v>46303.48493055555</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0115-26</t>
+          <t>SEC LMR BNM 0064-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -756,26 +776,26 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0115-26 DTG 061424Z OCT 262. BUOY RECOVERED BT</t>
+          <t>1. CANCEL SEC LMR BNM 0064-26 DTG 011740Z OCT 26 BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46302.45918981481</v>
+        <v>46303.48447916667</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0117-26</t>
+          <t>SEC LMR BNM 0059-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -789,29 +809,25 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF TROPICAL STORM ISAIAS, PROJECTED TO BECOME HURRICANE ISAIAS, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL WEATHER MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//102200Z OCT 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0059-26 DTG 121519Z SEP 26 BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46301.63203703704</v>
+        <v>46303.47424768518</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0058-26</t>
+          <t>CGD-H BNM 0116-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -834,21 +850,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0058-26 DTG 111759Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL CGD-H BNM 0116-26 DTG 061427Z OCT 262. BUOY RECOVERED BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46301.62190972222</v>
+        <v>46303.47325231481</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0116-26</t>
+          <t>CGD-H BNM 0115-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -867,34 +883,30 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-43-54.06N 096-58-39.60W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0115-26 DTG 061424Z OCT 262. BUOY RECOVERED BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46301.62096064815</v>
+        <v>46302.45918981481</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0115-26</t>
+          <t>CGD-H BNM 0117-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -910,76 +922,64 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-41-06.12N 97-00-12.00W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
+          <t>WITH THE APPROACH OF TROPICAL STORM ISAIAS, PROJECTED TO BECOME HURRICANE ISAIAS, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL WEATHER MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//102200Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46301.50265046296</v>
+        <v>46301.63203703704</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0066-26</t>
+          <t>SEC LMR BNM 0058-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>785</v>
-      </c>
-      <c r="K12" t="n">
-        <v>785</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>LMR 7851. DREDGE MIDWAY REQUESTS SLOW BELL NORTHBOUND AND SOUTHBOUND IVO MM 785 LMR.2. MARINERS ARE REQUESTED NOT TO MOOR UP BY THE PIPELINE.3. DREDGE MIDWAY CAN BE CONTACTED VIA VHF CHANNEL 13 OR 71.ALL MARINERS ARE REQUESTED TO TRANSIT THE AREA WITH CAUTION BT</t>
+          <t>1. CANCEL SEC LMR BNM 0058-26 DTG 111759Z SEP 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46300.76416666667</v>
+        <v>46301.62190972222</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0114-26</t>
+          <t>CGD-H BNM 0116-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1000,27 +1000,27 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010400Z NOV 26// BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-43-54.06N 096-58-39.60W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46300.76378472222</v>
+        <v>46301.62096064815</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0113-26</t>
+          <t>CGD-H BNM 0115-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1041,64 +1041,76 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>BETWEEN 07OCT2026 AND 18OCT2026, THE U.S. NAVY WILL CONDUCT DAILY UNEXPLODED ORDINANCE EXERCISES IN THE GULF OF AMERICA, NEAR APPROXIMATE POSITIONS 29-57-17.22N 086-03-03.36W AND 30-00-45.24N 085-44-27.30W. MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL CRAFT.CANCEL AT//190500Z OCT 26// BT</t>
+          <t>A YELLOW BUOY HAS BEEN REPORTED ADRIFT IN THE GULF OF AMERICA IN LAST KNOWN POSITION 26-41-06.12N 97-00-12.00W. MARINERS SHOULD TRANSIT WITH CAUTION AND REPORT ANY SIGHTINGS TO THE U.S. COAST GUARD.CANCEL AT//130500Z OCT 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46300.76337962963</v>
+        <v>46301.50265046296</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0112-26</t>
+          <t>SEC LMR BNM 0066-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>785</v>
+      </c>
+      <c r="K15" t="n">
+        <v>785</v>
+      </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0112-26 DTG 051544Z OCT 262. USAF MISSION CANCELLED. BT</t>
+          <t>LMR 7851. DREDGE MIDWAY REQUESTS SLOW BELL NORTHBOUND AND SOUTHBOUND IVO MM 785 LMR.2. MARINERS ARE REQUESTED NOT TO MOOR UP BY THE PIPELINE.3. DREDGE MIDWAY CAN BE CONTACTED VIA VHF CHANNEL 13 OR 71.ALL MARINERS ARE REQUESTED TO TRANSIT THE AREA WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46300.54696759259</v>
+        <v>46300.76416666667</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0112-26</t>
+          <t>CGD-H BNM 0114-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1125,21 +1137,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>ON 06OCT2026, BETWEEN 1300Z AND 1700Z, THE USAF WILL CONDUCT MUNITION LAUNCHES IN THE GULF OF AMERICA. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-16-50N 086-49-22W,30-10-09N 086-47-57W,29-51-08N 086-13-40W AND29-57-48N 086-32-54W.BACK-UP DATES INCLUDE 07OCT2026, 08OCT2026, 09OCT2026 AND 13OCT2026. MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//131800Z OCT 26// BT</t>
+          <t>UNMANNED SURFACE AND SUBSURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE IN THE GULF OF AMERICA INAN AREA BOUND BY APPROXIMATE POSITIONS:29-22-36.62N 087-24-41.36W,29-53-58.30N 086-55-55.00W AND 29-30-13.63N 086-32-57.29W.MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//010400Z NOV 26// BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46296.38649305556</v>
+        <v>46300.76378472222</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0062-26</t>
+          <t>CGD-H BNM 0113-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1158,90 +1170,66 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0062-26 DTG 282246Z SEP 26 BT</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>BETWEEN 07OCT2026 AND 18OCT2026, THE U.S. NAVY WILL CONDUCT DAILY UNEXPLODED ORDINANCE EXERCISES IN THE GULF OF AMERICA, NEAR APPROXIMATE POSITIONS 29-57-17.22N 086-03-03.36W AND 30-00-45.24N 085-44-27.30W. MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL CRAFT.CANCEL AT//190500Z OCT 26// BT</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"